<commit_message>
fix: export excell error
</commit_message>
<xml_diff>
--- a/packages/api-server/assets/evaluation-template.xlsx
+++ b/packages/api-server/assets/evaluation-template.xlsx
@@ -1,16 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27328"/>
-  <workbookPr defaultThemeVersion="166925"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Workspaces\Code\webProject\oss-evaluation-service\packages\api-server\excel\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\git\oss-evaluation-service\packages\api-server\assets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D6F7101A-7167-4824-A67D-F2A8C73DB53E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{8C35CFEB-34F0-4AA1-996E-72B6374757D4}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="2" r:id="rId1"/>
@@ -284,7 +283,7 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -302,18 +301,18 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="微软雅黑"/>
-      <family val="2"/>
+      <name val="宋体"/>
+      <family val="3"/>
       <charset val="134"/>
     </font>
     <font>
-      <b/>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="微软雅黑"/>
-      <family val="2"/>
+      <name val="宋体"/>
+      <family val="3"/>
       <charset val="134"/>
     </font>
   </fonts>
@@ -398,25 +397,25 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -732,356 +731,362 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BD3C2FFE-C49B-42B0-8643-73B7DCE3F264}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:E29"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultRowHeight="14" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="13.75" customWidth="1"/>
     <col min="2" max="2" width="13.25" customWidth="1"/>
-    <col min="3" max="3" width="26.375" customWidth="1"/>
+    <col min="3" max="3" width="26.33203125" customWidth="1"/>
     <col min="4" max="4" width="36" customWidth="1"/>
-    <col min="5" max="5" width="27.625" customWidth="1"/>
+    <col min="5" max="5" width="27.58203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="15" x14ac:dyDescent="0.2">
-      <c r="A1" s="2" t="s">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="2" t="s">
+      <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="2" t="s">
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="2" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="2" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:5" ht="16.5" x14ac:dyDescent="0.2">
-      <c r="A2" s="4" t="s">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A2" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="B2" s="1" t="s">
+      <c r="B2" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="C2" s="3" t="s">
+      <c r="C2" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="D2" s="1" t="s">
+      <c r="D2" s="3" t="s">
         <v>47</v>
       </c>
       <c r="E2" s="5" t="s">
         <v>65</v>
       </c>
     </row>
-    <row r="3" spans="1:5" ht="16.5" x14ac:dyDescent="0.2">
-      <c r="A3" s="4"/>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A3" s="2"/>
       <c r="B3" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="C3" s="3" t="s">
+      <c r="C3" s="4" t="s">
         <v>66</v>
       </c>
-      <c r="D3" s="1" t="s">
+      <c r="D3" s="3" t="s">
         <v>48</v>
       </c>
       <c r="E3" s="5"/>
     </row>
-    <row r="4" spans="1:5" ht="16.5" x14ac:dyDescent="0.2">
-      <c r="A4" s="4"/>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A4" s="2"/>
       <c r="B4" s="5"/>
-      <c r="C4" s="3" t="s">
+      <c r="C4" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="D4" s="1" t="s">
+      <c r="D4" s="3" t="s">
         <v>49</v>
       </c>
       <c r="E4" s="5"/>
     </row>
-    <row r="5" spans="1:5" ht="16.5" x14ac:dyDescent="0.2">
-      <c r="A5" s="4"/>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A5" s="2"/>
       <c r="B5" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="C5" s="3" t="s">
+      <c r="C5" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="D5" s="1"/>
+      <c r="D5" s="3"/>
       <c r="E5" s="5"/>
     </row>
-    <row r="6" spans="1:5" ht="16.5" x14ac:dyDescent="0.2">
-      <c r="A6" s="4"/>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A6" s="2"/>
       <c r="B6" s="5"/>
-      <c r="C6" s="3" t="s">
+      <c r="C6" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="D6" s="1"/>
+      <c r="D6" s="3"/>
       <c r="E6" s="5"/>
     </row>
-    <row r="7" spans="1:5" ht="16.5" x14ac:dyDescent="0.2">
-      <c r="A7" s="4" t="s">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A7" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="B7" s="1" t="s">
+      <c r="B7" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="C7" s="3" t="s">
+      <c r="C7" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="D7" s="1" t="s">
+      <c r="D7" s="3" t="s">
         <v>50</v>
       </c>
       <c r="E7" s="6" t="s">
         <v>64</v>
       </c>
     </row>
-    <row r="8" spans="1:5" ht="16.5" x14ac:dyDescent="0.2">
-      <c r="A8" s="4"/>
-      <c r="B8" s="1" t="s">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A8" s="2"/>
+      <c r="B8" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="C8" s="3" t="s">
+      <c r="C8" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="D8" s="1"/>
+      <c r="D8" s="3"/>
       <c r="E8" s="7"/>
     </row>
-    <row r="9" spans="1:5" ht="16.5" x14ac:dyDescent="0.2">
-      <c r="A9" s="4"/>
-      <c r="B9" s="1" t="s">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A9" s="2"/>
+      <c r="B9" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="C9" s="3" t="s">
+      <c r="C9" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="D9" s="1"/>
+      <c r="D9" s="3"/>
       <c r="E9" s="8"/>
     </row>
-    <row r="10" spans="1:5" ht="16.5" x14ac:dyDescent="0.2">
-      <c r="A10" s="4" t="s">
+    <row r="10" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A10" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="B10" s="1" t="s">
+      <c r="B10" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="C10" s="3" t="s">
+      <c r="C10" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="D10" s="1"/>
+      <c r="D10" s="3"/>
       <c r="E10" s="6" t="s">
         <v>62</v>
       </c>
     </row>
-    <row r="11" spans="1:5" ht="16.5" x14ac:dyDescent="0.2">
-      <c r="A11" s="4"/>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A11" s="2"/>
       <c r="B11" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="C11" s="3" t="s">
+      <c r="C11" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="D11" s="1"/>
+      <c r="D11" s="3"/>
       <c r="E11" s="7"/>
     </row>
-    <row r="12" spans="1:5" ht="16.5" x14ac:dyDescent="0.2">
-      <c r="A12" s="4"/>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A12" s="2"/>
       <c r="B12" s="5"/>
-      <c r="C12" s="3" t="s">
+      <c r="C12" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="D12" s="1"/>
+      <c r="D12" s="3"/>
       <c r="E12" s="8"/>
     </row>
-    <row r="13" spans="1:5" ht="16.5" x14ac:dyDescent="0.2">
-      <c r="A13" s="4" t="s">
+    <row r="13" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A13" s="2" t="s">
         <v>46</v>
       </c>
       <c r="B13" s="5" t="s">
         <v>26</v>
       </c>
-      <c r="C13" s="3" t="s">
+      <c r="C13" s="4" t="s">
         <v>27</v>
       </c>
-      <c r="D13" s="1" t="s">
+      <c r="D13" s="3" t="s">
         <v>51</v>
       </c>
       <c r="E13" s="6" t="s">
         <v>63</v>
       </c>
     </row>
-    <row r="14" spans="1:5" ht="16.5" x14ac:dyDescent="0.2">
-      <c r="A14" s="4"/>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A14" s="2"/>
       <c r="B14" s="5"/>
-      <c r="C14" s="3" t="s">
+      <c r="C14" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="D14" s="1"/>
+      <c r="D14" s="3"/>
       <c r="E14" s="7"/>
     </row>
-    <row r="15" spans="1:5" ht="16.5" x14ac:dyDescent="0.2">
-      <c r="A15" s="4"/>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A15" s="2"/>
       <c r="B15" s="5"/>
-      <c r="C15" s="3" t="s">
+      <c r="C15" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="D15" s="1" t="s">
+      <c r="D15" s="3" t="s">
         <v>52</v>
       </c>
       <c r="E15" s="7"/>
     </row>
-    <row r="16" spans="1:5" ht="16.5" x14ac:dyDescent="0.2">
-      <c r="A16" s="4"/>
+    <row r="16" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A16" s="2"/>
       <c r="B16" s="5"/>
-      <c r="C16" s="3" t="s">
+      <c r="C16" s="4" t="s">
         <v>30</v>
       </c>
-      <c r="D16" s="1" t="s">
+      <c r="D16" s="3" t="s">
         <v>53</v>
       </c>
       <c r="E16" s="7"/>
     </row>
-    <row r="17" spans="1:5" ht="16.5" x14ac:dyDescent="0.2">
-      <c r="A17" s="4"/>
+    <row r="17" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A17" s="2"/>
       <c r="B17" s="5"/>
-      <c r="C17" s="3" t="s">
+      <c r="C17" s="4" t="s">
         <v>31</v>
       </c>
-      <c r="D17" s="1"/>
+      <c r="D17" s="3"/>
       <c r="E17" s="7"/>
     </row>
-    <row r="18" spans="1:5" ht="16.5" x14ac:dyDescent="0.2">
-      <c r="A18" s="4"/>
+    <row r="18" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A18" s="2"/>
       <c r="B18" s="5" t="s">
         <v>43</v>
       </c>
-      <c r="C18" s="3" t="s">
+      <c r="C18" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="D18" s="1" t="s">
+      <c r="D18" s="3" t="s">
         <v>54</v>
       </c>
       <c r="E18" s="7"/>
     </row>
-    <row r="19" spans="1:5" ht="16.5" x14ac:dyDescent="0.2">
-      <c r="A19" s="4"/>
+    <row r="19" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A19" s="2"/>
       <c r="B19" s="5"/>
-      <c r="C19" s="3" t="s">
+      <c r="C19" s="4" t="s">
         <v>33</v>
       </c>
-      <c r="D19" s="1"/>
+      <c r="D19" s="3"/>
       <c r="E19" s="7"/>
     </row>
-    <row r="20" spans="1:5" ht="16.5" x14ac:dyDescent="0.2">
-      <c r="A20" s="4"/>
+    <row r="20" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A20" s="2"/>
       <c r="B20" s="5"/>
-      <c r="C20" s="3" t="s">
+      <c r="C20" s="4" t="s">
         <v>34</v>
       </c>
-      <c r="D20" s="1"/>
+      <c r="D20" s="3"/>
       <c r="E20" s="7"/>
     </row>
-    <row r="21" spans="1:5" ht="16.5" x14ac:dyDescent="0.2">
-      <c r="A21" s="4"/>
+    <row r="21" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A21" s="2"/>
       <c r="B21" s="5"/>
-      <c r="C21" s="3" t="s">
+      <c r="C21" s="4" t="s">
         <v>35</v>
       </c>
-      <c r="D21" s="1" t="s">
+      <c r="D21" s="3" t="s">
         <v>55</v>
       </c>
       <c r="E21" s="7"/>
     </row>
-    <row r="22" spans="1:5" ht="16.5" x14ac:dyDescent="0.2">
-      <c r="A22" s="4"/>
+    <row r="22" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A22" s="2"/>
       <c r="B22" s="5"/>
-      <c r="C22" s="3" t="s">
+      <c r="C22" s="4" t="s">
         <v>36</v>
       </c>
-      <c r="D22" s="1" t="s">
+      <c r="D22" s="3" t="s">
         <v>56</v>
       </c>
       <c r="E22" s="7"/>
     </row>
-    <row r="23" spans="1:5" ht="16.5" x14ac:dyDescent="0.2">
-      <c r="A23" s="4"/>
+    <row r="23" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A23" s="2"/>
       <c r="B23" s="5"/>
-      <c r="C23" s="3" t="s">
+      <c r="C23" s="4" t="s">
         <v>37</v>
       </c>
-      <c r="D23" s="1" t="s">
+      <c r="D23" s="3" t="s">
         <v>57</v>
       </c>
       <c r="E23" s="7"/>
     </row>
-    <row r="24" spans="1:5" ht="16.5" x14ac:dyDescent="0.2">
-      <c r="A24" s="4"/>
+    <row r="24" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A24" s="2"/>
       <c r="B24" s="5"/>
-      <c r="C24" s="3" t="s">
+      <c r="C24" s="4" t="s">
         <v>38</v>
       </c>
-      <c r="D24" s="1" t="s">
+      <c r="D24" s="3" t="s">
         <v>58</v>
       </c>
       <c r="E24" s="7"/>
     </row>
-    <row r="25" spans="1:5" ht="16.5" x14ac:dyDescent="0.2">
-      <c r="A25" s="4"/>
+    <row r="25" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A25" s="2"/>
       <c r="B25" s="5"/>
-      <c r="C25" s="3" t="s">
+      <c r="C25" s="4" t="s">
         <v>39</v>
       </c>
-      <c r="D25" s="1" t="s">
+      <c r="D25" s="3" t="s">
         <v>59</v>
       </c>
       <c r="E25" s="7"/>
     </row>
-    <row r="26" spans="1:5" ht="16.5" x14ac:dyDescent="0.2">
-      <c r="A26" s="4"/>
+    <row r="26" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A26" s="2"/>
       <c r="B26" s="5"/>
-      <c r="C26" s="3" t="s">
+      <c r="C26" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="D26" s="1" t="s">
+      <c r="D26" s="3" t="s">
         <v>60</v>
       </c>
       <c r="E26" s="7"/>
     </row>
-    <row r="27" spans="1:5" ht="16.5" x14ac:dyDescent="0.2">
-      <c r="A27" s="4"/>
+    <row r="27" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A27" s="2"/>
       <c r="B27" s="5"/>
-      <c r="C27" s="3" t="s">
+      <c r="C27" s="4" t="s">
         <v>41</v>
       </c>
-      <c r="D27" s="1"/>
+      <c r="D27" s="3"/>
       <c r="E27" s="7"/>
     </row>
-    <row r="28" spans="1:5" ht="16.5" x14ac:dyDescent="0.2">
-      <c r="A28" s="4"/>
+    <row r="28" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A28" s="2"/>
       <c r="B28" s="5"/>
-      <c r="C28" s="3" t="s">
+      <c r="C28" s="4" t="s">
         <v>42</v>
       </c>
-      <c r="D28" s="1"/>
+      <c r="D28" s="3"/>
       <c r="E28" s="7"/>
     </row>
-    <row r="29" spans="1:5" ht="16.5" x14ac:dyDescent="0.2">
-      <c r="A29" s="4"/>
-      <c r="B29" s="1" t="s">
+    <row r="29" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A29" s="2"/>
+      <c r="B29" s="3" t="s">
         <v>45</v>
       </c>
-      <c r="C29" s="3" t="s">
+      <c r="C29" s="4" t="s">
         <v>44</v>
       </c>
-      <c r="D29" s="1" t="s">
+      <c r="D29" s="3" t="s">
         <v>61</v>
       </c>
       <c r="E29" s="8"/>
     </row>
   </sheetData>
   <mergeCells count="13">
+    <mergeCell ref="A2:A6"/>
+    <mergeCell ref="E2:E6"/>
+    <mergeCell ref="B3:B4"/>
+    <mergeCell ref="B5:B6"/>
+    <mergeCell ref="A7:A9"/>
+    <mergeCell ref="E7:E9"/>
     <mergeCell ref="A10:A12"/>
     <mergeCell ref="E10:E12"/>
     <mergeCell ref="B11:B12"/>
@@ -1089,12 +1094,6 @@
     <mergeCell ref="B13:B17"/>
     <mergeCell ref="E13:E29"/>
     <mergeCell ref="B18:B28"/>
-    <mergeCell ref="A2:A6"/>
-    <mergeCell ref="E2:E6"/>
-    <mergeCell ref="B3:B4"/>
-    <mergeCell ref="B5:B6"/>
-    <mergeCell ref="A7:A9"/>
-    <mergeCell ref="E7:E9"/>
   </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
refactor(export): merge performance api into project api
merge performance api into project api
</commit_message>
<xml_diff>
--- a/packages/api-server/assets/evaluation-template.xlsx
+++ b/packages/api-server/assets/evaluation-template.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\DayDream\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Workspaces\Code\webProject\oss-evaluation-service\packages\api-server\assets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{9EA836E4-2B80-48B4-9E5B-2CDCB4ED5DA5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6AE871CE-D843-45D2-9F37-FBF329EC020F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{156AEBF6-8089-4DBA-97A4-A673309B8D23}"/>
   </bookViews>
@@ -518,10 +518,6 @@
     <t>开发者满意度</t>
   </si>
   <si>
-    <t>&lt;%~data._data_.satisfactionExport%&gt;</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
     <t>&lt;%=data._data_.evaluation.functionScore%&gt;</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
@@ -666,10 +662,6 @@
     <t>打包大小</t>
   </si>
   <si>
-    <t>&lt;%~data._data_.gzipSize%&gt; kB</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
     <t>生态</t>
   </si>
   <si>
@@ -770,6 +762,14 @@
   </si>
   <si>
     <t>&lt;%~data._data_.evaluation.recentReleasesCount%&gt;</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>&lt;%~data._data_.performanceInfo.gzipSize%&gt; kB</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>&lt;%=data._data_.satisfactionExport%&gt;</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
 </sst>
@@ -903,25 +903,25 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1275,95 +1275,95 @@
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A2" s="2" t="s">
+      <c r="A2" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="B2" s="3" t="s">
+      <c r="B2" s="7" t="s">
         <v>6</v>
       </c>
-      <c r="C2" s="4" t="s">
+      <c r="C2" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="D2" s="5" t="s">
+      <c r="D2" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="E2" s="3" t="s">
+      <c r="E2" s="7" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A3" s="6"/>
-      <c r="B3" s="7"/>
-      <c r="C3" s="4" t="s">
+      <c r="A3" s="5"/>
+      <c r="B3" s="8"/>
+      <c r="C3" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="D3" s="5" t="s">
+      <c r="D3" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="E3" s="7"/>
+      <c r="E3" s="8"/>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A4" s="6"/>
-      <c r="B4" s="7"/>
-      <c r="C4" s="4" t="s">
+      <c r="A4" s="5"/>
+      <c r="B4" s="8"/>
+      <c r="C4" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="D4" s="5" t="s">
+      <c r="D4" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="E4" s="7"/>
+      <c r="E4" s="8"/>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A5" s="6"/>
-      <c r="B5" s="7"/>
-      <c r="C5" s="4" t="s">
+      <c r="A5" s="5"/>
+      <c r="B5" s="8"/>
+      <c r="C5" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="D5" s="5" t="s">
+      <c r="D5" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="E5" s="7"/>
+      <c r="E5" s="8"/>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A6" s="6"/>
-      <c r="B6" s="7"/>
-      <c r="C6" s="4" t="s">
+      <c r="A6" s="5"/>
+      <c r="B6" s="8"/>
+      <c r="C6" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="D6" s="5" t="s">
+      <c r="D6" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="E6" s="7"/>
+      <c r="E6" s="8"/>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A7" s="6"/>
-      <c r="B7" s="7"/>
-      <c r="C7" s="4" t="s">
+      <c r="A7" s="5"/>
+      <c r="B7" s="8"/>
+      <c r="C7" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="D7" s="5" t="s">
+      <c r="D7" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="E7" s="7"/>
+      <c r="E7" s="8"/>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A8" s="6"/>
-      <c r="B8" s="7"/>
-      <c r="C8" s="4" t="s">
+      <c r="A8" s="5"/>
+      <c r="B8" s="8"/>
+      <c r="C8" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="D8" s="5" t="s">
+      <c r="D8" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="E8" s="7"/>
+      <c r="E8" s="8"/>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A9" s="8"/>
+      <c r="A9" s="6"/>
       <c r="B9" s="9"/>
-      <c r="C9" s="4" t="s">
+      <c r="C9" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="D9" s="5" t="s">
+      <c r="D9" s="3" t="s">
         <v>23</v>
       </c>
       <c r="E9" s="9"/>
@@ -1375,355 +1375,355 @@
       <c r="B10" s="11" t="s">
         <v>25</v>
       </c>
-      <c r="C10" s="4" t="s">
+      <c r="C10" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="D10" s="5" t="s">
+      <c r="D10" s="3" t="s">
+        <v>104</v>
+      </c>
+      <c r="E10" s="11" t="s">
         <v>27</v>
-      </c>
-      <c r="E10" s="11" t="s">
-        <v>28</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A11" s="10"/>
       <c r="B11" s="11"/>
-      <c r="C11" s="4" t="s">
+      <c r="C11" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="D11" s="3" t="s">
         <v>29</v>
-      </c>
-      <c r="D11" s="5" t="s">
-        <v>30</v>
       </c>
       <c r="E11" s="11"/>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A12" s="10"/>
       <c r="B12" s="11"/>
-      <c r="C12" s="4" t="s">
+      <c r="C12" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="D12" s="3" t="s">
         <v>31</v>
       </c>
-      <c r="D12" s="5" t="s">
+      <c r="E12" s="11"/>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A13" s="5" t="s">
         <v>32</v>
       </c>
-      <c r="E12" s="11"/>
-    </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A13" s="6" t="s">
+      <c r="B13" s="7" t="s">
         <v>33</v>
       </c>
-      <c r="B13" s="3" t="s">
+      <c r="C13" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="C13" s="4" t="s">
+      <c r="D13" s="3" t="s">
         <v>35</v>
       </c>
-      <c r="D13" s="5" t="s">
+      <c r="E13" s="8" t="s">
         <v>36</v>
       </c>
-      <c r="E13" s="7" t="s">
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A14" s="5"/>
+      <c r="B14" s="8"/>
+      <c r="C14" s="2" t="s">
         <v>37</v>
       </c>
-    </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A14" s="6"/>
-      <c r="B14" s="7"/>
-      <c r="C14" s="4" t="s">
+      <c r="D14" s="3" t="s">
         <v>38</v>
       </c>
-      <c r="D14" s="5" t="s">
+      <c r="E14" s="8"/>
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A15" s="5"/>
+      <c r="B15" s="8"/>
+      <c r="C15" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="E14" s="7"/>
-    </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A15" s="6"/>
-      <c r="B15" s="7"/>
-      <c r="C15" s="4" t="s">
+      <c r="D15" s="3" t="s">
         <v>40</v>
       </c>
-      <c r="D15" s="5" t="s">
+      <c r="E15" s="8"/>
+    </row>
+    <row r="16" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A16" s="5"/>
+      <c r="B16" s="8"/>
+      <c r="C16" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="D16" s="3" t="s">
         <v>41</v>
       </c>
-      <c r="E15" s="7"/>
-    </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A16" s="6"/>
-      <c r="B16" s="7"/>
-      <c r="C16" s="4" t="s">
-        <v>22</v>
-      </c>
-      <c r="D16" s="5" t="s">
+      <c r="E16" s="8"/>
+    </row>
+    <row r="17" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A17" s="5"/>
+      <c r="B17" s="8"/>
+      <c r="C17" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="E16" s="7"/>
-    </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A17" s="6"/>
-      <c r="B17" s="7"/>
-      <c r="C17" s="4" t="s">
+      <c r="D17" s="3" t="s">
         <v>43</v>
       </c>
-      <c r="D17" s="5" t="s">
+      <c r="E17" s="8"/>
+    </row>
+    <row r="18" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A18" s="5"/>
+      <c r="B18" s="8"/>
+      <c r="C18" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="E17" s="7"/>
-    </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A18" s="6"/>
-      <c r="B18" s="7"/>
-      <c r="C18" s="4" t="s">
+      <c r="D18" s="3" t="s">
         <v>45</v>
       </c>
-      <c r="D18" s="5" t="s">
+      <c r="E18" s="8"/>
+    </row>
+    <row r="19" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A19" s="5"/>
+      <c r="B19" s="8"/>
+      <c r="C19" s="2" t="s">
         <v>46</v>
       </c>
-      <c r="E18" s="7"/>
-    </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A19" s="6"/>
-      <c r="B19" s="7"/>
-      <c r="C19" s="4" t="s">
+      <c r="D19" s="3" t="s">
         <v>47</v>
       </c>
-      <c r="D19" s="5" t="s">
+      <c r="E19" s="8"/>
+    </row>
+    <row r="20" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A20" s="5"/>
+      <c r="B20" s="8"/>
+      <c r="C20" s="2" t="s">
         <v>48</v>
       </c>
-      <c r="E19" s="7"/>
-    </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A20" s="6"/>
-      <c r="B20" s="7"/>
-      <c r="C20" s="4" t="s">
+      <c r="D20" s="3" t="s">
         <v>49</v>
       </c>
-      <c r="D20" s="5" t="s">
+      <c r="E20" s="8"/>
+    </row>
+    <row r="21" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A21" s="5"/>
+      <c r="B21" s="8"/>
+      <c r="C21" s="2" t="s">
         <v>50</v>
       </c>
-      <c r="E20" s="7"/>
-    </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A21" s="6"/>
-      <c r="B21" s="7"/>
-      <c r="C21" s="4" t="s">
+      <c r="D21" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="E21" s="8"/>
+    </row>
+    <row r="22" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A22" s="5"/>
+      <c r="B22" s="8"/>
+      <c r="C22" s="2" t="s">
         <v>51</v>
       </c>
-      <c r="D21" s="5" t="s">
-        <v>48</v>
-      </c>
-      <c r="E21" s="7"/>
-    </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A22" s="6"/>
-      <c r="B22" s="7"/>
-      <c r="C22" s="4" t="s">
+      <c r="D22" s="3" t="s">
         <v>52</v>
       </c>
-      <c r="D22" s="5" t="s">
+      <c r="E22" s="8"/>
+    </row>
+    <row r="23" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A23" s="5"/>
+      <c r="B23" s="8"/>
+      <c r="C23" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="E22" s="7"/>
-    </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A23" s="6"/>
-      <c r="B23" s="7"/>
-      <c r="C23" s="4" t="s">
+      <c r="D23" s="3" t="s">
         <v>54</v>
       </c>
-      <c r="D23" s="5" t="s">
+      <c r="E23" s="8"/>
+    </row>
+    <row r="24" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A24" s="5"/>
+      <c r="B24" s="8"/>
+      <c r="C24" s="2" t="s">
         <v>55</v>
       </c>
-      <c r="E23" s="7"/>
-    </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A24" s="6"/>
-      <c r="B24" s="7"/>
-      <c r="C24" s="4" t="s">
+      <c r="D24" s="3" t="s">
         <v>56</v>
       </c>
-      <c r="D24" s="5" t="s">
+      <c r="E24" s="8"/>
+    </row>
+    <row r="25" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A25" s="5"/>
+      <c r="B25" s="9"/>
+      <c r="C25" s="2" t="s">
         <v>57</v>
       </c>
-      <c r="E24" s="7"/>
-    </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A25" s="6"/>
-      <c r="B25" s="9"/>
-      <c r="C25" s="4" t="s">
+      <c r="D25" s="3" t="s">
         <v>58</v>
       </c>
-      <c r="D25" s="5" t="s">
+      <c r="E25" s="8"/>
+    </row>
+    <row r="26" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A26" s="5"/>
+      <c r="B26" s="7" t="s">
         <v>59</v>
       </c>
-      <c r="E25" s="7"/>
-    </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A26" s="6"/>
-      <c r="B26" s="3" t="s">
+      <c r="C26" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="C26" s="4" t="s">
+      <c r="D26" s="3" t="s">
         <v>61</v>
       </c>
-      <c r="D26" s="5" t="s">
+      <c r="E26" s="8"/>
+    </row>
+    <row r="27" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A27" s="5"/>
+      <c r="B27" s="8"/>
+      <c r="C27" s="2" t="s">
         <v>62</v>
       </c>
-      <c r="E26" s="7"/>
-    </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A27" s="6"/>
-      <c r="B27" s="7"/>
-      <c r="C27" s="4" t="s">
+      <c r="D27" s="3" t="s">
         <v>63</v>
       </c>
-      <c r="D27" s="5" t="s">
+      <c r="E27" s="8"/>
+    </row>
+    <row r="28" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A28" s="5"/>
+      <c r="B28" s="8"/>
+      <c r="C28" s="2" t="s">
         <v>64</v>
       </c>
-      <c r="E27" s="7"/>
-    </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A28" s="6"/>
-      <c r="B28" s="7"/>
-      <c r="C28" s="4" t="s">
+      <c r="D28" s="3" t="s">
         <v>65</v>
       </c>
-      <c r="D28" s="5" t="s">
+      <c r="E28" s="8"/>
+    </row>
+    <row r="29" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A29" s="6"/>
+      <c r="B29" s="9"/>
+      <c r="C29" s="2" t="s">
         <v>66</v>
       </c>
-      <c r="E28" s="7"/>
-    </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A29" s="8"/>
-      <c r="B29" s="9"/>
-      <c r="C29" s="4" t="s">
+      <c r="D29" s="3" t="s">
         <v>67</v>
-      </c>
-      <c r="D29" s="5" t="s">
-        <v>68</v>
       </c>
       <c r="E29" s="9"/>
     </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A30" s="10" t="s">
+        <v>68</v>
+      </c>
+      <c r="B30" s="3" t="s">
         <v>69</v>
       </c>
-      <c r="B30" s="5" t="s">
+      <c r="C30" s="2" t="s">
         <v>70</v>
       </c>
-      <c r="C30" s="4" t="s">
-        <v>71</v>
-      </c>
-      <c r="D30" s="5" t="s">
+      <c r="D30" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="E30" s="3" t="s">
+      <c r="E30" s="7" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="31" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A31" s="10"/>
-      <c r="B31" s="5" t="s">
+      <c r="B31" s="3" t="s">
+        <v>71</v>
+      </c>
+      <c r="C31" s="2" t="s">
         <v>72</v>
       </c>
-      <c r="C31" s="4" t="s">
-        <v>73</v>
-      </c>
-      <c r="D31" s="5" t="s">
-        <v>74</v>
-      </c>
-      <c r="E31" s="7"/>
+      <c r="D31" s="3" t="s">
+        <v>103</v>
+      </c>
+      <c r="E31" s="8"/>
     </row>
     <row r="32" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A32" s="10" t="s">
+        <v>73</v>
+      </c>
+      <c r="B32" s="7" t="s">
+        <v>74</v>
+      </c>
+      <c r="C32" s="2" t="s">
         <v>75</v>
       </c>
-      <c r="B32" s="3" t="s">
+      <c r="D32" s="3" t="s">
         <v>76</v>
       </c>
-      <c r="C32" s="4" t="s">
+      <c r="E32" s="11" t="s">
         <v>77</v>
-      </c>
-      <c r="D32" s="5" t="s">
-        <v>78</v>
-      </c>
-      <c r="E32" s="11" t="s">
-        <v>79</v>
       </c>
     </row>
     <row r="33" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A33" s="10"/>
-      <c r="B33" s="7"/>
-      <c r="C33" s="4" t="s">
-        <v>80</v>
-      </c>
-      <c r="D33" s="5" t="s">
-        <v>81</v>
+      <c r="B33" s="8"/>
+      <c r="C33" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="D33" s="3" t="s">
+        <v>79</v>
       </c>
       <c r="E33" s="11"/>
     </row>
     <row r="34" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A34" s="10"/>
-      <c r="B34" s="7"/>
-      <c r="C34" s="4" t="s">
-        <v>82</v>
-      </c>
-      <c r="D34" s="5" t="s">
-        <v>83</v>
+      <c r="B34" s="8"/>
+      <c r="C34" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="D34" s="3" t="s">
+        <v>81</v>
       </c>
       <c r="E34" s="11"/>
     </row>
     <row r="35" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A35" s="10"/>
       <c r="B35" s="9"/>
-      <c r="C35" s="4" t="s">
-        <v>84</v>
-      </c>
-      <c r="D35" s="5" t="s">
-        <v>85</v>
+      <c r="C35" s="2" t="s">
+        <v>82</v>
+      </c>
+      <c r="D35" s="3" t="s">
+        <v>83</v>
       </c>
       <c r="E35" s="11"/>
     </row>
     <row r="36" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A36" s="10"/>
       <c r="B36" s="11" t="s">
+        <v>84</v>
+      </c>
+      <c r="C36" s="2" t="s">
+        <v>85</v>
+      </c>
+      <c r="D36" s="3" t="s">
         <v>86</v>
-      </c>
-      <c r="C36" s="4" t="s">
-        <v>87</v>
-      </c>
-      <c r="D36" s="5" t="s">
-        <v>88</v>
       </c>
       <c r="E36" s="11"/>
     </row>
     <row r="37" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A37" s="10"/>
       <c r="B37" s="11"/>
-      <c r="C37" s="4" t="s">
-        <v>89</v>
-      </c>
-      <c r="D37" s="5" t="s">
-        <v>90</v>
+      <c r="C37" s="2" t="s">
+        <v>87</v>
+      </c>
+      <c r="D37" s="3" t="s">
+        <v>88</v>
       </c>
       <c r="E37" s="11"/>
     </row>
     <row r="38" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A38" s="10"/>
       <c r="B38" s="11"/>
-      <c r="C38" s="4" t="s">
-        <v>91</v>
-      </c>
-      <c r="D38" s="5" t="s">
-        <v>92</v>
+      <c r="C38" s="2" t="s">
+        <v>89</v>
+      </c>
+      <c r="D38" s="3" t="s">
+        <v>90</v>
       </c>
       <c r="E38" s="11"/>
     </row>
     <row r="39" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A39" s="10"/>
       <c r="B39" s="11"/>
-      <c r="C39" s="4" t="s">
-        <v>93</v>
-      </c>
-      <c r="D39" s="5" t="s">
+      <c r="C39" s="2" t="s">
+        <v>91</v>
+      </c>
+      <c r="D39" s="3" t="s">
         <v>9</v>
       </c>
       <c r="E39" s="11"/>
@@ -1731,57 +1731,57 @@
     <row r="40" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A40" s="10"/>
       <c r="B40" s="11" t="s">
+        <v>92</v>
+      </c>
+      <c r="C40" s="2" t="s">
+        <v>93</v>
+      </c>
+      <c r="D40" s="3" t="s">
         <v>94</v>
-      </c>
-      <c r="C40" s="4" t="s">
-        <v>95</v>
-      </c>
-      <c r="D40" s="5" t="s">
-        <v>96</v>
       </c>
       <c r="E40" s="11"/>
     </row>
     <row r="41" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A41" s="10"/>
       <c r="B41" s="11"/>
-      <c r="C41" s="4" t="s">
-        <v>97</v>
-      </c>
-      <c r="D41" s="5" t="s">
-        <v>98</v>
+      <c r="C41" s="2" t="s">
+        <v>95</v>
+      </c>
+      <c r="D41" s="3" t="s">
+        <v>96</v>
       </c>
       <c r="E41" s="11"/>
     </row>
     <row r="42" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A42" s="10"/>
       <c r="B42" s="11"/>
-      <c r="C42" s="4" t="s">
-        <v>99</v>
-      </c>
-      <c r="D42" s="5" t="s">
-        <v>100</v>
+      <c r="C42" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="D42" s="3" t="s">
+        <v>98</v>
       </c>
       <c r="E42" s="11"/>
     </row>
     <row r="43" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A43" s="10"/>
       <c r="B43" s="11"/>
-      <c r="C43" s="4" t="s">
-        <v>101</v>
-      </c>
-      <c r="D43" s="5" t="s">
-        <v>102</v>
+      <c r="C43" s="2" t="s">
+        <v>99</v>
+      </c>
+      <c r="D43" s="3" t="s">
+        <v>100</v>
       </c>
       <c r="E43" s="11"/>
     </row>
     <row r="44" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A44" s="10"/>
       <c r="B44" s="11"/>
-      <c r="C44" s="4" t="s">
-        <v>103</v>
-      </c>
-      <c r="D44" s="5" t="s">
-        <v>104</v>
+      <c r="C44" s="2" t="s">
+        <v>101</v>
+      </c>
+      <c r="D44" s="3" t="s">
+        <v>102</v>
       </c>
       <c r="E44" s="11"/>
     </row>

</xml_diff>

<commit_message>
feat: add homepage for software detail
</commit_message>
<xml_diff>
--- a/packages/api-server/assets/evaluation-template.xlsx
+++ b/packages/api-server/assets/evaluation-template.xlsx
@@ -1,21 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27425"/>
-  <workbookPr defaultThemeVersion="166925"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\DayDream\Desktop\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\git\oss-evaluation-service\packages\api-server\assets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{9EA836E4-2B80-48B4-9E5B-2CDCB4ED5DA5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{156AEBF6-8089-4DBA-97A4-A673309B8D23}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="181029"/>
+  <calcPr calcId="152511"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -25,12 +24,12 @@
 </file>
 
 <file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <authors>
     <author>DayDream</author>
   </authors>
   <commentList>
-    <comment ref="C10" authorId="0" shapeId="0" xr:uid="{7B295FC2-BA71-46C8-9067-C29C5833A7FE}">
+    <comment ref="C11" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -44,7 +43,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="C12" authorId="0" shapeId="0" xr:uid="{70B60FA2-3FE6-4C82-AFA8-1A42E59E3C7D}">
+    <comment ref="C13" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -58,7 +57,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="B13" authorId="0" shapeId="0" xr:uid="{A2259C0E-70DE-4E8E-990E-6CBB7BF1CAEC}">
+    <comment ref="B14" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -82,7 +81,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="C13" authorId="0" shapeId="0" xr:uid="{B598CB59-F274-423D-9DCE-BBA72B60022A}">
+    <comment ref="C14" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -96,7 +95,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="C14" authorId="0" shapeId="0" xr:uid="{F1D200CE-C6BE-4A65-8BE9-0A763552CBAD}">
+    <comment ref="C15" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -120,7 +119,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="C15" authorId="0" shapeId="0" xr:uid="{9C97B50E-CAE5-4480-A6BE-D01BF2A5DC15}">
+    <comment ref="C16" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -144,7 +143,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="C16" authorId="0" shapeId="0" xr:uid="{AF57E2B5-C4A5-4929-83E1-C172F6DF2D01}">
+    <comment ref="C17" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -168,7 +167,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="C17" authorId="0" shapeId="0" xr:uid="{5799924F-51F5-436F-BF6C-ED819709FCF1}">
+    <comment ref="C18" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -192,7 +191,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="C18" authorId="0" shapeId="0" xr:uid="{83C3A96B-513B-4BE5-A2B9-E301B15F6C8B}">
+    <comment ref="C19" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -216,7 +215,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="C19" authorId="0" shapeId="0" xr:uid="{AAE3B769-9E29-42ED-BF42-E9795A6D1E07}">
+    <comment ref="C20" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -240,7 +239,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="C20" authorId="0" shapeId="0" xr:uid="{77C3FCF8-37E7-4001-919F-BB2B7F354888}">
+    <comment ref="C21" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -264,7 +263,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="C21" authorId="0" shapeId="0" xr:uid="{176F5CDE-FB55-4232-A553-8F5F4F71EC10}">
+    <comment ref="C22" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -288,7 +287,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="C22" authorId="0" shapeId="0" xr:uid="{FB23BBBA-1C1C-41EE-AE78-0EAB750B68A0}">
+    <comment ref="C23" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -302,7 +301,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="C23" authorId="0" shapeId="0" xr:uid="{70629A5A-3ADA-4B71-A682-D4ACEF4313D2}">
+    <comment ref="C24" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -326,7 +325,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="C24" authorId="0" shapeId="0" xr:uid="{F5399C77-147C-45AB-AB6D-59696D224CFB}">
+    <comment ref="C25" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -350,7 +349,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="C25" authorId="0" shapeId="0" xr:uid="{76F325EF-1145-4991-9576-4FDFA01259F6}">
+    <comment ref="C26" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -374,7 +373,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="C35" authorId="0" shapeId="0" xr:uid="{77B3997A-0EFC-4039-953C-230C868E1D8C}">
+    <comment ref="C36" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -388,7 +387,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="C36" authorId="0" shapeId="0" xr:uid="{24D8232D-31D1-45A7-8A16-BEA6348576BD}">
+    <comment ref="C37" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -402,7 +401,7 @@
         </r>
       </text>
     </comment>
-    <comment ref="C37" authorId="0" shapeId="0" xr:uid="{C6F2D215-8A56-4375-8C6B-ABF73DC7C1F2}">
+    <comment ref="C38" authorId="0" shapeId="0">
       <text>
         <r>
           <rPr>
@@ -431,7 +430,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="110" uniqueCount="105">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="112" uniqueCount="105">
   <si>
     <t>维度</t>
   </si>
@@ -457,9 +456,6 @@
     <t>名称</t>
   </si>
   <si>
-    <t>&lt;%=data._data_.evaluation.projectName%&gt;</t>
-  </si>
-  <si>
     <t>/</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
@@ -467,10 +463,6 @@
     <t>技术栈分类</t>
   </si>
   <si>
-    <t>&lt;%=data._data_.evaluation.techStack%&gt;</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
     <t>简介</t>
   </si>
   <si>
@@ -480,10 +472,6 @@
     <t>官网地址</t>
   </si>
   <si>
-    <t>&lt;%=data._data_.githubProjects.homePage%&gt;</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
     <t>Stars</t>
   </si>
   <si>
@@ -529,10 +517,6 @@
     <t>代码量</t>
   </si>
   <si>
-    <t>&lt;%~data._data_.codeLines%&gt; KL</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
     <t>文档最佳实践</t>
   </si>
   <si>
@@ -690,17 +674,9 @@
     <t>Star数量</t>
   </si>
   <si>
-    <t>&lt;%~data._data_.evaluation.stargazersCount%&gt;</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
     <t>Fork数量</t>
   </si>
   <si>
-    <t>&lt;%~data._data_.evaluation.forksCount%&gt;</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
     <t>巴士系数</t>
   </si>
   <si>
@@ -770,13 +746,37 @@
   </si>
   <si>
     <t>&lt;%~data._data_.evaluation.recentReleasesCount%&gt;</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>&lt;%=data._data_.homePage%&gt;</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Fork</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>&lt;%~data._data_.fork%&gt;</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>&lt;%=data._data_.techStack%&gt;</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>&lt;%=data._data_.repoName%&gt;</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>&lt;%~data._data_.codeLines%&gt; kl</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -896,17 +896,11 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -915,13 +909,22 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1246,18 +1249,18 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8AD8815F-8FA3-405C-8D93-992A405E03EE}">
-  <dimension ref="A1:E44"/>
-  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:E45"/>
+  <sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="16.25" customWidth="1"/>
-    <col min="2" max="2" width="18.875" customWidth="1"/>
-    <col min="3" max="3" width="33.5" customWidth="1"/>
-    <col min="4" max="4" width="39.375" customWidth="1"/>
-    <col min="5" max="5" width="24.625" customWidth="1"/>
+    <col min="1" max="1" width="16.21875" customWidth="1"/>
+    <col min="2" max="2" width="18.88671875" customWidth="1"/>
+    <col min="3" max="3" width="33.44140625" customWidth="1"/>
+    <col min="4" max="4" width="39.33203125" customWidth="1"/>
+    <col min="5" max="5" width="24.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:5" ht="14.4" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1274,536 +1277,547 @@
         <v>4</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A2" s="2" t="s">
+    <row r="2" spans="1:5" ht="14.4" x14ac:dyDescent="0.25">
+      <c r="A2" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="B2" s="3" t="s">
+      <c r="B2" s="8" t="s">
         <v>6</v>
       </c>
-      <c r="C2" s="4" t="s">
+      <c r="C2" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="D2" s="5" t="s">
+      <c r="D2" s="3" t="s">
+        <v>103</v>
+      </c>
+      <c r="E2" s="8" t="s">
         <v>8</v>
       </c>
-      <c r="E2" s="3" t="s">
+    </row>
+    <row r="3" spans="1:5" ht="14.4" x14ac:dyDescent="0.25">
+      <c r="A3" s="6"/>
+      <c r="B3" s="9"/>
+      <c r="C3" s="2" t="s">
         <v>9</v>
       </c>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A3" s="6"/>
-      <c r="B3" s="7"/>
-      <c r="C3" s="4" t="s">
+      <c r="D3" s="3" t="s">
+        <v>102</v>
+      </c>
+      <c r="E3" s="9"/>
+    </row>
+    <row r="4" spans="1:5" ht="14.4" x14ac:dyDescent="0.25">
+      <c r="A4" s="6"/>
+      <c r="B4" s="9"/>
+      <c r="C4" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="D3" s="5" t="s">
+      <c r="D4" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="E3" s="7"/>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A4" s="6"/>
-      <c r="B4" s="7"/>
-      <c r="C4" s="4" t="s">
+      <c r="E4" s="9"/>
+    </row>
+    <row r="5" spans="1:5" ht="14.4" x14ac:dyDescent="0.25">
+      <c r="A5" s="6"/>
+      <c r="B5" s="9"/>
+      <c r="C5" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="D4" s="5" t="s">
+      <c r="D5" s="3" t="s">
+        <v>99</v>
+      </c>
+      <c r="E5" s="9"/>
+    </row>
+    <row r="6" spans="1:5" ht="14.4" x14ac:dyDescent="0.25">
+      <c r="A6" s="6"/>
+      <c r="B6" s="9"/>
+      <c r="C6" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="E4" s="7"/>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A5" s="6"/>
-      <c r="B5" s="7"/>
-      <c r="C5" s="4" t="s">
+      <c r="D6" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="D5" s="5" t="s">
+      <c r="E6" s="9"/>
+    </row>
+    <row r="7" spans="1:5" ht="14.4" x14ac:dyDescent="0.25">
+      <c r="A7" s="6"/>
+      <c r="B7" s="9"/>
+      <c r="C7" s="2" t="s">
+        <v>100</v>
+      </c>
+      <c r="D7" s="4" t="s">
+        <v>101</v>
+      </c>
+      <c r="E7" s="9"/>
+    </row>
+    <row r="8" spans="1:5" ht="14.4" x14ac:dyDescent="0.25">
+      <c r="A8" s="6"/>
+      <c r="B8" s="9"/>
+      <c r="C8" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="E5" s="7"/>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A6" s="6"/>
-      <c r="B6" s="7"/>
-      <c r="C6" s="4" t="s">
+      <c r="D8" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="D6" s="5" t="s">
+      <c r="E8" s="9"/>
+    </row>
+    <row r="9" spans="1:5" ht="14.4" x14ac:dyDescent="0.25">
+      <c r="A9" s="6"/>
+      <c r="B9" s="9"/>
+      <c r="C9" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="E6" s="7"/>
-    </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A7" s="6"/>
-      <c r="B7" s="7"/>
-      <c r="C7" s="4" t="s">
+      <c r="D9" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="D7" s="5" t="s">
+      <c r="E9" s="9"/>
+    </row>
+    <row r="10" spans="1:5" ht="14.4" x14ac:dyDescent="0.25">
+      <c r="A10" s="7"/>
+      <c r="B10" s="10"/>
+      <c r="C10" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="E7" s="7"/>
-    </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A8" s="6"/>
-      <c r="B8" s="7"/>
-      <c r="C8" s="4" t="s">
+      <c r="D10" s="3" t="s">
         <v>20</v>
       </c>
-      <c r="D8" s="5" t="s">
+      <c r="E10" s="10"/>
+    </row>
+    <row r="11" spans="1:5" ht="14.4" x14ac:dyDescent="0.25">
+      <c r="A11" s="11" t="s">
         <v>21</v>
       </c>
-      <c r="E8" s="7"/>
-    </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A9" s="8"/>
-      <c r="B9" s="9"/>
-      <c r="C9" s="4" t="s">
+      <c r="B11" s="12" t="s">
         <v>22</v>
       </c>
-      <c r="D9" s="5" t="s">
+      <c r="C11" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="E9" s="9"/>
-    </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A10" s="10" t="s">
+      <c r="D11" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="B10" s="11" t="s">
+      <c r="E11" s="12" t="s">
         <v>25</v>
       </c>
-      <c r="C10" s="4" t="s">
+    </row>
+    <row r="12" spans="1:5" ht="14.4" x14ac:dyDescent="0.25">
+      <c r="A12" s="11"/>
+      <c r="B12" s="12"/>
+      <c r="C12" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="D10" s="5" t="s">
+      <c r="D12" s="3" t="s">
+        <v>104</v>
+      </c>
+      <c r="E12" s="12"/>
+    </row>
+    <row r="13" spans="1:5" ht="14.4" x14ac:dyDescent="0.25">
+      <c r="A13" s="11"/>
+      <c r="B13" s="12"/>
+      <c r="C13" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="E10" s="11" t="s">
+      <c r="D13" s="3" t="s">
         <v>28</v>
       </c>
-    </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A11" s="10"/>
-      <c r="B11" s="11"/>
-      <c r="C11" s="4" t="s">
+      <c r="E13" s="12"/>
+    </row>
+    <row r="14" spans="1:5" ht="14.4" x14ac:dyDescent="0.25">
+      <c r="A14" s="6" t="s">
         <v>29</v>
       </c>
-      <c r="D11" s="5" t="s">
+      <c r="B14" s="8" t="s">
         <v>30</v>
       </c>
-      <c r="E11" s="11"/>
-    </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A12" s="10"/>
-      <c r="B12" s="11"/>
-      <c r="C12" s="4" t="s">
+      <c r="C14" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="D12" s="5" t="s">
+      <c r="D14" s="3" t="s">
         <v>32</v>
       </c>
-      <c r="E12" s="11"/>
-    </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A13" s="6" t="s">
+      <c r="E14" s="9" t="s">
         <v>33</v>
       </c>
-      <c r="B13" s="3" t="s">
+    </row>
+    <row r="15" spans="1:5" ht="14.4" x14ac:dyDescent="0.25">
+      <c r="A15" s="6"/>
+      <c r="B15" s="9"/>
+      <c r="C15" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="C13" s="4" t="s">
+      <c r="D15" s="3" t="s">
         <v>35</v>
       </c>
-      <c r="D13" s="5" t="s">
+      <c r="E15" s="9"/>
+    </row>
+    <row r="16" spans="1:5" ht="14.4" x14ac:dyDescent="0.25">
+      <c r="A16" s="6"/>
+      <c r="B16" s="9"/>
+      <c r="C16" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="E13" s="7" t="s">
+      <c r="D16" s="3" t="s">
         <v>37</v>
       </c>
-    </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A14" s="6"/>
-      <c r="B14" s="7"/>
-      <c r="C14" s="4" t="s">
+      <c r="E16" s="9"/>
+    </row>
+    <row r="17" spans="1:5" ht="14.4" x14ac:dyDescent="0.25">
+      <c r="A17" s="6"/>
+      <c r="B17" s="9"/>
+      <c r="C17" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="D17" s="3" t="s">
         <v>38</v>
       </c>
-      <c r="D14" s="5" t="s">
+      <c r="E17" s="9"/>
+    </row>
+    <row r="18" spans="1:5" ht="14.4" x14ac:dyDescent="0.25">
+      <c r="A18" s="6"/>
+      <c r="B18" s="9"/>
+      <c r="C18" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="E14" s="7"/>
-    </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A15" s="6"/>
-      <c r="B15" s="7"/>
-      <c r="C15" s="4" t="s">
+      <c r="D18" s="3" t="s">
         <v>40</v>
       </c>
-      <c r="D15" s="5" t="s">
+      <c r="E18" s="9"/>
+    </row>
+    <row r="19" spans="1:5" ht="14.4" x14ac:dyDescent="0.25">
+      <c r="A19" s="6"/>
+      <c r="B19" s="9"/>
+      <c r="C19" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="E15" s="7"/>
-    </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A16" s="6"/>
-      <c r="B16" s="7"/>
-      <c r="C16" s="4" t="s">
-        <v>22</v>
-      </c>
-      <c r="D16" s="5" t="s">
+      <c r="D19" s="3" t="s">
         <v>42</v>
       </c>
-      <c r="E16" s="7"/>
-    </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A17" s="6"/>
-      <c r="B17" s="7"/>
-      <c r="C17" s="4" t="s">
+      <c r="E19" s="9"/>
+    </row>
+    <row r="20" spans="1:5" ht="14.4" x14ac:dyDescent="0.25">
+      <c r="A20" s="6"/>
+      <c r="B20" s="9"/>
+      <c r="C20" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="D17" s="5" t="s">
+      <c r="D20" s="3" t="s">
         <v>44</v>
       </c>
-      <c r="E17" s="7"/>
-    </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A18" s="6"/>
-      <c r="B18" s="7"/>
-      <c r="C18" s="4" t="s">
+      <c r="E20" s="9"/>
+    </row>
+    <row r="21" spans="1:5" ht="14.4" x14ac:dyDescent="0.25">
+      <c r="A21" s="6"/>
+      <c r="B21" s="9"/>
+      <c r="C21" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="D18" s="5" t="s">
+      <c r="D21" s="3" t="s">
         <v>46</v>
       </c>
-      <c r="E18" s="7"/>
-    </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A19" s="6"/>
-      <c r="B19" s="7"/>
-      <c r="C19" s="4" t="s">
+      <c r="E21" s="9"/>
+    </row>
+    <row r="22" spans="1:5" ht="14.4" x14ac:dyDescent="0.25">
+      <c r="A22" s="6"/>
+      <c r="B22" s="9"/>
+      <c r="C22" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="D19" s="5" t="s">
+      <c r="D22" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="E22" s="9"/>
+    </row>
+    <row r="23" spans="1:5" ht="14.4" x14ac:dyDescent="0.25">
+      <c r="A23" s="6"/>
+      <c r="B23" s="9"/>
+      <c r="C23" s="2" t="s">
         <v>48</v>
       </c>
-      <c r="E19" s="7"/>
-    </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A20" s="6"/>
-      <c r="B20" s="7"/>
-      <c r="C20" s="4" t="s">
+      <c r="D23" s="3" t="s">
         <v>49</v>
       </c>
-      <c r="D20" s="5" t="s">
+      <c r="E23" s="9"/>
+    </row>
+    <row r="24" spans="1:5" ht="14.4" x14ac:dyDescent="0.25">
+      <c r="A24" s="6"/>
+      <c r="B24" s="9"/>
+      <c r="C24" s="2" t="s">
         <v>50</v>
       </c>
-      <c r="E20" s="7"/>
-    </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A21" s="6"/>
-      <c r="B21" s="7"/>
-      <c r="C21" s="4" t="s">
+      <c r="D24" s="3" t="s">
         <v>51</v>
       </c>
-      <c r="D21" s="5" t="s">
-        <v>48</v>
-      </c>
-      <c r="E21" s="7"/>
-    </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A22" s="6"/>
-      <c r="B22" s="7"/>
-      <c r="C22" s="4" t="s">
-        <v>52</v>
-      </c>
-      <c r="D22" s="5" t="s">
-        <v>53</v>
-      </c>
-      <c r="E22" s="7"/>
-    </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A23" s="6"/>
-      <c r="B23" s="7"/>
-      <c r="C23" s="4" t="s">
-        <v>54</v>
-      </c>
-      <c r="D23" s="5" t="s">
-        <v>55</v>
-      </c>
-      <c r="E23" s="7"/>
-    </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A24" s="6"/>
-      <c r="B24" s="7"/>
-      <c r="C24" s="4" t="s">
-        <v>56</v>
-      </c>
-      <c r="D24" s="5" t="s">
-        <v>57</v>
-      </c>
-      <c r="E24" s="7"/>
-    </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="E24" s="9"/>
+    </row>
+    <row r="25" spans="1:5" ht="14.4" x14ac:dyDescent="0.25">
       <c r="A25" s="6"/>
       <c r="B25" s="9"/>
-      <c r="C25" s="4" t="s">
+      <c r="C25" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="D25" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="E25" s="9"/>
+    </row>
+    <row r="26" spans="1:5" ht="14.4" x14ac:dyDescent="0.25">
+      <c r="A26" s="6"/>
+      <c r="B26" s="10"/>
+      <c r="C26" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="D26" s="3" t="s">
+        <v>55</v>
+      </c>
+      <c r="E26" s="9"/>
+    </row>
+    <row r="27" spans="1:5" ht="14.4" x14ac:dyDescent="0.25">
+      <c r="A27" s="6"/>
+      <c r="B27" s="8" t="s">
+        <v>56</v>
+      </c>
+      <c r="C27" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="D27" s="3" t="s">
         <v>58</v>
       </c>
-      <c r="D25" s="5" t="s">
+      <c r="E27" s="9"/>
+    </row>
+    <row r="28" spans="1:5" ht="14.4" x14ac:dyDescent="0.25">
+      <c r="A28" s="6"/>
+      <c r="B28" s="9"/>
+      <c r="C28" s="2" t="s">
         <v>59</v>
       </c>
-      <c r="E25" s="7"/>
-    </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A26" s="6"/>
-      <c r="B26" s="3" t="s">
+      <c r="D28" s="3" t="s">
         <v>60</v>
       </c>
-      <c r="C26" s="4" t="s">
+      <c r="E28" s="9"/>
+    </row>
+    <row r="29" spans="1:5" ht="14.4" x14ac:dyDescent="0.25">
+      <c r="A29" s="6"/>
+      <c r="B29" s="9"/>
+      <c r="C29" s="2" t="s">
         <v>61</v>
       </c>
-      <c r="D26" s="5" t="s">
+      <c r="D29" s="3" t="s">
         <v>62</v>
       </c>
-      <c r="E26" s="7"/>
-    </row>
-    <row r="27" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A27" s="6"/>
-      <c r="B27" s="7"/>
-      <c r="C27" s="4" t="s">
+      <c r="E29" s="9"/>
+    </row>
+    <row r="30" spans="1:5" ht="14.4" x14ac:dyDescent="0.25">
+      <c r="A30" s="7"/>
+      <c r="B30" s="10"/>
+      <c r="C30" s="2" t="s">
         <v>63</v>
       </c>
-      <c r="D27" s="5" t="s">
+      <c r="D30" s="3" t="s">
         <v>64</v>
       </c>
-      <c r="E27" s="7"/>
-    </row>
-    <row r="28" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A28" s="6"/>
-      <c r="B28" s="7"/>
-      <c r="C28" s="4" t="s">
+      <c r="E30" s="10"/>
+    </row>
+    <row r="31" spans="1:5" ht="14.4" x14ac:dyDescent="0.25">
+      <c r="A31" s="11" t="s">
         <v>65</v>
       </c>
-      <c r="D28" s="5" t="s">
+      <c r="B31" s="3" t="s">
         <v>66</v>
       </c>
-      <c r="E28" s="7"/>
-    </row>
-    <row r="29" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A29" s="8"/>
-      <c r="B29" s="9"/>
-      <c r="C29" s="4" t="s">
+      <c r="C31" s="2" t="s">
         <v>67</v>
       </c>
-      <c r="D29" s="5" t="s">
+      <c r="D31" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="E31" s="8" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="32" spans="1:5" ht="14.4" x14ac:dyDescent="0.25">
+      <c r="A32" s="11"/>
+      <c r="B32" s="3" t="s">
         <v>68</v>
       </c>
-      <c r="E29" s="9"/>
-    </row>
-    <row r="30" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A30" s="10" t="s">
+      <c r="C32" s="2" t="s">
         <v>69</v>
       </c>
-      <c r="B30" s="5" t="s">
+      <c r="D32" s="3" t="s">
         <v>70</v>
       </c>
-      <c r="C30" s="4" t="s">
+      <c r="E32" s="9"/>
+    </row>
+    <row r="33" spans="1:5" ht="14.4" x14ac:dyDescent="0.25">
+      <c r="A33" s="11" t="s">
         <v>71</v>
       </c>
-      <c r="D30" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="E30" s="3" t="s">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="31" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A31" s="10"/>
-      <c r="B31" s="5" t="s">
+      <c r="B33" s="8" t="s">
         <v>72</v>
       </c>
-      <c r="C31" s="4" t="s">
+      <c r="C33" s="2" t="s">
         <v>73</v>
       </c>
-      <c r="D31" s="5" t="s">
+      <c r="D33" s="3" t="s">
         <v>74</v>
       </c>
-      <c r="E31" s="7"/>
-    </row>
-    <row r="32" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A32" s="10" t="s">
+      <c r="E33" s="12" t="s">
         <v>75</v>
       </c>
-      <c r="B32" s="3" t="s">
+    </row>
+    <row r="34" spans="1:5" ht="14.4" x14ac:dyDescent="0.25">
+      <c r="A34" s="11"/>
+      <c r="B34" s="9"/>
+      <c r="C34" s="2" t="s">
         <v>76</v>
       </c>
-      <c r="C32" s="4" t="s">
+      <c r="D34" s="4" t="s">
+        <v>14</v>
+      </c>
+      <c r="E34" s="12"/>
+    </row>
+    <row r="35" spans="1:5" ht="14.4" x14ac:dyDescent="0.25">
+      <c r="A35" s="11"/>
+      <c r="B35" s="9"/>
+      <c r="C35" s="2" t="s">
         <v>77</v>
       </c>
-      <c r="D32" s="5" t="s">
+      <c r="D35" s="4" t="s">
+        <v>101</v>
+      </c>
+      <c r="E35" s="12"/>
+    </row>
+    <row r="36" spans="1:5" ht="14.4" x14ac:dyDescent="0.25">
+      <c r="A36" s="11"/>
+      <c r="B36" s="10"/>
+      <c r="C36" s="2" t="s">
         <v>78</v>
       </c>
-      <c r="E32" s="11" t="s">
+      <c r="D36" s="3" t="s">
         <v>79</v>
       </c>
-    </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A33" s="10"/>
-      <c r="B33" s="7"/>
-      <c r="C33" s="4" t="s">
+      <c r="E36" s="12"/>
+    </row>
+    <row r="37" spans="1:5" ht="14.4" x14ac:dyDescent="0.25">
+      <c r="A37" s="11"/>
+      <c r="B37" s="12" t="s">
         <v>80</v>
       </c>
-      <c r="D33" s="5" t="s">
+      <c r="C37" s="2" t="s">
         <v>81</v>
       </c>
-      <c r="E33" s="11"/>
-    </row>
-    <row r="34" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A34" s="10"/>
-      <c r="B34" s="7"/>
-      <c r="C34" s="4" t="s">
+      <c r="D37" s="3" t="s">
         <v>82</v>
       </c>
-      <c r="D34" s="5" t="s">
+      <c r="E37" s="12"/>
+    </row>
+    <row r="38" spans="1:5" ht="14.4" x14ac:dyDescent="0.25">
+      <c r="A38" s="11"/>
+      <c r="B38" s="12"/>
+      <c r="C38" s="2" t="s">
         <v>83</v>
       </c>
-      <c r="E34" s="11"/>
-    </row>
-    <row r="35" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A35" s="10"/>
-      <c r="B35" s="9"/>
-      <c r="C35" s="4" t="s">
+      <c r="D38" s="3" t="s">
         <v>84</v>
       </c>
-      <c r="D35" s="5" t="s">
+      <c r="E38" s="12"/>
+    </row>
+    <row r="39" spans="1:5" ht="14.4" x14ac:dyDescent="0.25">
+      <c r="A39" s="11"/>
+      <c r="B39" s="12"/>
+      <c r="C39" s="2" t="s">
         <v>85</v>
       </c>
-      <c r="E35" s="11"/>
-    </row>
-    <row r="36" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A36" s="10"/>
-      <c r="B36" s="11" t="s">
+      <c r="D39" s="3" t="s">
         <v>86</v>
       </c>
-      <c r="C36" s="4" t="s">
+      <c r="E39" s="12"/>
+    </row>
+    <row r="40" spans="1:5" ht="14.4" x14ac:dyDescent="0.25">
+      <c r="A40" s="11"/>
+      <c r="B40" s="12"/>
+      <c r="C40" s="2" t="s">
         <v>87</v>
       </c>
-      <c r="D36" s="5" t="s">
+      <c r="D40" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="E40" s="12"/>
+    </row>
+    <row r="41" spans="1:5" ht="14.4" x14ac:dyDescent="0.25">
+      <c r="A41" s="11"/>
+      <c r="B41" s="12" t="s">
         <v>88</v>
       </c>
-      <c r="E36" s="11"/>
-    </row>
-    <row r="37" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A37" s="10"/>
-      <c r="B37" s="11"/>
-      <c r="C37" s="4" t="s">
+      <c r="C41" s="2" t="s">
         <v>89</v>
       </c>
-      <c r="D37" s="5" t="s">
+      <c r="D41" s="3" t="s">
         <v>90</v>
       </c>
-      <c r="E37" s="11"/>
-    </row>
-    <row r="38" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A38" s="10"/>
-      <c r="B38" s="11"/>
-      <c r="C38" s="4" t="s">
+      <c r="E41" s="12"/>
+    </row>
+    <row r="42" spans="1:5" ht="14.4" x14ac:dyDescent="0.25">
+      <c r="A42" s="11"/>
+      <c r="B42" s="12"/>
+      <c r="C42" s="2" t="s">
         <v>91</v>
       </c>
-      <c r="D38" s="5" t="s">
+      <c r="D42" s="3" t="s">
         <v>92</v>
       </c>
-      <c r="E38" s="11"/>
-    </row>
-    <row r="39" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A39" s="10"/>
-      <c r="B39" s="11"/>
-      <c r="C39" s="4" t="s">
+      <c r="E42" s="12"/>
+    </row>
+    <row r="43" spans="1:5" ht="14.4" x14ac:dyDescent="0.25">
+      <c r="A43" s="11"/>
+      <c r="B43" s="12"/>
+      <c r="C43" s="2" t="s">
         <v>93</v>
       </c>
-      <c r="D39" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="E39" s="11"/>
-    </row>
-    <row r="40" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A40" s="10"/>
-      <c r="B40" s="11" t="s">
+      <c r="D43" s="3" t="s">
         <v>94</v>
       </c>
-      <c r="C40" s="4" t="s">
+      <c r="E43" s="12"/>
+    </row>
+    <row r="44" spans="1:5" ht="14.4" x14ac:dyDescent="0.25">
+      <c r="A44" s="11"/>
+      <c r="B44" s="12"/>
+      <c r="C44" s="2" t="s">
         <v>95</v>
       </c>
-      <c r="D40" s="5" t="s">
+      <c r="D44" s="3" t="s">
         <v>96</v>
       </c>
-      <c r="E40" s="11"/>
-    </row>
-    <row r="41" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A41" s="10"/>
-      <c r="B41" s="11"/>
-      <c r="C41" s="4" t="s">
+      <c r="E44" s="12"/>
+    </row>
+    <row r="45" spans="1:5" ht="14.4" x14ac:dyDescent="0.25">
+      <c r="A45" s="11"/>
+      <c r="B45" s="12"/>
+      <c r="C45" s="2" t="s">
         <v>97</v>
       </c>
-      <c r="D41" s="5" t="s">
+      <c r="D45" s="3" t="s">
         <v>98</v>
       </c>
-      <c r="E41" s="11"/>
-    </row>
-    <row r="42" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A42" s="10"/>
-      <c r="B42" s="11"/>
-      <c r="C42" s="4" t="s">
-        <v>99</v>
-      </c>
-      <c r="D42" s="5" t="s">
-        <v>100</v>
-      </c>
-      <c r="E42" s="11"/>
-    </row>
-    <row r="43" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A43" s="10"/>
-      <c r="B43" s="11"/>
-      <c r="C43" s="4" t="s">
-        <v>101</v>
-      </c>
-      <c r="D43" s="5" t="s">
-        <v>102</v>
-      </c>
-      <c r="E43" s="11"/>
-    </row>
-    <row r="44" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A44" s="10"/>
-      <c r="B44" s="11"/>
-      <c r="C44" s="4" t="s">
-        <v>103</v>
-      </c>
-      <c r="D44" s="5" t="s">
-        <v>104</v>
-      </c>
-      <c r="E44" s="11"/>
+      <c r="E45" s="12"/>
     </row>
   </sheetData>
   <mergeCells count="17">
-    <mergeCell ref="A32:A44"/>
-    <mergeCell ref="B32:B35"/>
-    <mergeCell ref="E32:E44"/>
-    <mergeCell ref="B36:B39"/>
-    <mergeCell ref="B40:B44"/>
-    <mergeCell ref="A13:A29"/>
-    <mergeCell ref="B13:B25"/>
-    <mergeCell ref="E13:E29"/>
-    <mergeCell ref="B26:B29"/>
-    <mergeCell ref="A30:A31"/>
-    <mergeCell ref="E30:E31"/>
-    <mergeCell ref="A2:A9"/>
-    <mergeCell ref="B2:B9"/>
-    <mergeCell ref="E2:E9"/>
-    <mergeCell ref="A10:A12"/>
-    <mergeCell ref="B10:B12"/>
-    <mergeCell ref="E10:E12"/>
+    <mergeCell ref="A33:A45"/>
+    <mergeCell ref="B33:B36"/>
+    <mergeCell ref="E33:E45"/>
+    <mergeCell ref="B37:B40"/>
+    <mergeCell ref="B41:B45"/>
+    <mergeCell ref="A14:A30"/>
+    <mergeCell ref="B14:B26"/>
+    <mergeCell ref="E14:E30"/>
+    <mergeCell ref="B27:B30"/>
+    <mergeCell ref="A31:A32"/>
+    <mergeCell ref="E31:E32"/>
+    <mergeCell ref="A2:A10"/>
+    <mergeCell ref="B2:B10"/>
+    <mergeCell ref="E2:E10"/>
+    <mergeCell ref="A11:A13"/>
+    <mergeCell ref="B11:B13"/>
+    <mergeCell ref="E11:E13"/>
   </mergeCells>
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
fix(export): Fixed the problem of no main package export error
Fixed the problem of no main package export error
</commit_message>
<xml_diff>
--- a/packages/api-server/assets/evaluation-template.xlsx
+++ b/packages/api-server/assets/evaluation-template.xlsx
@@ -1,15 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
-  <workbookPr/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27531"/>
+  <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\git\oss-evaluation-service\packages\api-server\assets\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Workspaces\Code\webProject\oss-evaluation-service\packages\api-server\assets\"/>
     </mc:Choice>
   </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2A556DD7-DC56-42BD-B103-0F4391A39E1D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -405,87 +406,88 @@
     <t>&lt;%~_data_.scorecard.pinnedDependencies%&gt;</t>
   </si>
   <si>
+    <t>&lt;%= _data_?.sonarCloudScan?.maintainabilityRating || 'N/A' %&gt;</t>
+  </si>
+  <si>
+    <t>&lt;%= _data_?.sonarCloudScan?.securityRating || 'N/A' %&gt;</t>
+  </si>
+  <si>
+    <t>&lt;%= _data_?.sonarCloudScan?.securityReviewRating || 'N/A' %&gt;</t>
+  </si>
+  <si>
+    <t>&lt;%~_data_.evaluation.ecologyScore%&gt;</t>
+  </si>
+  <si>
+    <t>&lt;%~_data_.evaluation.busFactor%&gt;</t>
+  </si>
+  <si>
+    <t>&lt;%~_data_.evaluation.openrank%&gt;</t>
+  </si>
+  <si>
+    <t>&lt;%~_data_.evaluation.criticalityScore%&gt;</t>
+  </si>
+  <si>
+    <t>&lt;%~_data_.contributors%&gt;</t>
+  </si>
+  <si>
+    <t>&lt;%~_data_.dependentRepositories%&gt;</t>
+  </si>
+  <si>
+    <t>&lt;%~_data_.evaluation.commitFrequency%&gt;</t>
+  </si>
+  <si>
+    <t>&lt;%~_data_.evaluation.orgCount%&gt;</t>
+  </si>
+  <si>
+    <t>&lt;%~_data_.evaluation.commentFrequency%&gt;</t>
+  </si>
+  <si>
+    <t>&lt;%~_data_.evaluation.updatedIssuesCount%&gt;</t>
+  </si>
+  <si>
+    <t>&lt;%~_data_.evaluation.closedIssuesCount%&gt;</t>
+  </si>
+  <si>
+    <t>&lt;%~_data_.evaluation.recentReleasesCount%&gt;</t>
+  </si>
+  <si>
+    <t>&lt;%~_data_.scorecard.codeReview%&gt;</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Scorecard</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>包大小(kB)</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>周下载量(k)</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>&lt;%~_data_.evaluation.npmDownloads/1000%&gt;</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
     <t>&lt;%= _data_?.sonarCloudScan?.reliabilityRating || 'N/A' %&gt;</t>
-  </si>
-  <si>
-    <t>&lt;%= _data_?.sonarCloudScan?.maintainabilityRating || 'N/A' %&gt;</t>
-  </si>
-  <si>
-    <t>&lt;%= _data_?.sonarCloudScan?.securityRating || 'N/A' %&gt;</t>
-  </si>
-  <si>
-    <t>&lt;%= _data_?.sonarCloudScan?.securityReviewRating || 'N/A' %&gt;</t>
-  </si>
-  <si>
-    <t>&lt;%~_data_.evaluation.ecologyScore%&gt;</t>
-  </si>
-  <si>
-    <t>&lt;%~_data_.evaluation.busFactor%&gt;</t>
-  </si>
-  <si>
-    <t>&lt;%~_data_.evaluation.openrank%&gt;</t>
-  </si>
-  <si>
-    <t>&lt;%~_data_.evaluation.criticalityScore%&gt;</t>
-  </si>
-  <si>
-    <t>&lt;%~_data_.contributors%&gt;</t>
-  </si>
-  <si>
-    <t>&lt;%~_data_.dependentRepositories%&gt;</t>
-  </si>
-  <si>
-    <t>&lt;%~_data_.evaluation.commitFrequency%&gt;</t>
-  </si>
-  <si>
-    <t>&lt;%~_data_.evaluation.orgCount%&gt;</t>
-  </si>
-  <si>
-    <t>&lt;%~_data_.evaluation.commentFrequency%&gt;</t>
-  </si>
-  <si>
-    <t>&lt;%~_data_.evaluation.updatedIssuesCount%&gt;</t>
-  </si>
-  <si>
-    <t>&lt;%~_data_.evaluation.closedIssuesCount%&gt;</t>
-  </si>
-  <si>
-    <t>&lt;%~_data_.evaluation.recentReleasesCount%&gt;</t>
-  </si>
-  <si>
-    <t>&lt;%~_data_.scorecard.codeReview%&gt;</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>Scorecard</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>包大小(kB)</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>&lt;%~_data_.gzipSize/1024%&gt;</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>周下载量(k)</t>
-    <phoneticPr fontId="2" type="noConversion"/>
-  </si>
-  <si>
-    <t>&lt;%~_data_.evaluation.npmDownloads/1000%&gt;</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>&lt;%~_data_?.gzipSize/1024 || 'N/A' %&gt;</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="4">
     <numFmt numFmtId="176" formatCode="0.00_);[Red]\(0.00\)"/>
     <numFmt numFmtId="177" formatCode="0.00_ "/>
     <numFmt numFmtId="178" formatCode="0_);[Red]\(0\)"/>
-    <numFmt numFmtId="181" formatCode="0.0_);[Red]\(0.0\)"/>
+    <numFmt numFmtId="179" formatCode="0.0_);[Red]\(0.0\)"/>
   </numFmts>
   <fonts count="5" x14ac:knownFonts="1">
     <font>
@@ -602,7 +604,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -618,7 +620,7 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="176" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -627,42 +629,36 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="177" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
     <xf numFmtId="178" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="179" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="176" fontId="4" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -672,7 +668,7 @@
     <xf numFmtId="176" fontId="4" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="181" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -988,43 +984,43 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:G47"/>
-  <sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="13.33203125" style="1" customWidth="1"/>
+    <col min="1" max="1" width="13.375" style="1" customWidth="1"/>
     <col min="2" max="2" width="14" customWidth="1"/>
-    <col min="3" max="3" width="24.6640625" customWidth="1"/>
-    <col min="4" max="4" width="28.88671875" style="2" customWidth="1"/>
-    <col min="5" max="5" width="29.44140625" style="2" customWidth="1"/>
-    <col min="6" max="6" width="34.109375" style="2" customWidth="1"/>
+    <col min="3" max="3" width="24.625" customWidth="1"/>
+    <col min="4" max="4" width="28.875" style="2" customWidth="1"/>
+    <col min="5" max="5" width="62" style="2" customWidth="1"/>
+    <col min="6" max="6" width="34.125" style="2" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="14.4" x14ac:dyDescent="0.25">
-      <c r="A1" s="11" t="s">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A1" s="10" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="11" t="s">
+      <c r="B1" s="10" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="11" t="s">
+      <c r="C1" s="10" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="11" t="s">
+      <c r="D1" s="10" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="11" t="s">
+      <c r="E1" s="10" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="11" t="s">
+      <c r="F1" s="10" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:7" ht="14.4" x14ac:dyDescent="0.25">
-      <c r="A2" s="14" t="s">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A2" s="16" t="s">
         <v>6</v>
       </c>
-      <c r="B2" s="17" t="s">
+      <c r="B2" s="13" t="s">
         <v>7</v>
       </c>
       <c r="C2" s="3" t="s">
@@ -1034,14 +1030,14 @@
       <c r="E2" s="5" t="s">
         <v>93</v>
       </c>
-      <c r="F2" s="20" t="s">
+      <c r="F2" s="18" t="s">
         <v>7</v>
       </c>
       <c r="G2" s="2"/>
     </row>
-    <row r="3" spans="1:7" ht="14.4" x14ac:dyDescent="0.25">
-      <c r="A3" s="15"/>
-      <c r="B3" s="18"/>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A3" s="21"/>
+      <c r="B3" s="14"/>
       <c r="C3" s="3" t="s">
         <v>9</v>
       </c>
@@ -1049,23 +1045,23 @@
       <c r="E3" s="5" t="s">
         <v>94</v>
       </c>
-      <c r="F3" s="21"/>
-    </row>
-    <row r="4" spans="1:7" ht="14.4" x14ac:dyDescent="0.25">
-      <c r="A4" s="15"/>
-      <c r="B4" s="18"/>
+      <c r="F3" s="19"/>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A4" s="21"/>
+      <c r="B4" s="14"/>
       <c r="C4" s="3" t="s">
         <v>10</v>
       </c>
       <c r="D4" s="4"/>
-      <c r="E4" s="12" t="s">
+      <c r="E4" s="4" t="s">
         <v>95</v>
       </c>
-      <c r="F4" s="21"/>
-    </row>
-    <row r="5" spans="1:7" ht="14.4" x14ac:dyDescent="0.25">
-      <c r="A5" s="15"/>
-      <c r="B5" s="18"/>
+      <c r="F4" s="19"/>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A5" s="21"/>
+      <c r="B5" s="14"/>
       <c r="C5" s="3" t="s">
         <v>11</v>
       </c>
@@ -1073,35 +1069,35 @@
       <c r="E5" s="5" t="s">
         <v>96</v>
       </c>
-      <c r="F5" s="21"/>
-    </row>
-    <row r="6" spans="1:7" ht="14.4" x14ac:dyDescent="0.25">
-      <c r="A6" s="15"/>
-      <c r="B6" s="18"/>
+      <c r="F5" s="19"/>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A6" s="21"/>
+      <c r="B6" s="14"/>
       <c r="C6" s="3" t="s">
         <v>12</v>
       </c>
       <c r="D6" s="4"/>
-      <c r="E6" s="13" t="s">
+      <c r="E6" s="11" t="s">
         <v>97</v>
       </c>
-      <c r="F6" s="21"/>
-    </row>
-    <row r="7" spans="1:7" ht="14.4" x14ac:dyDescent="0.25">
-      <c r="A7" s="15"/>
-      <c r="B7" s="18"/>
+      <c r="F6" s="19"/>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A7" s="21"/>
+      <c r="B7" s="14"/>
       <c r="C7" s="3" t="s">
         <v>13</v>
       </c>
       <c r="D7" s="4"/>
-      <c r="E7" s="13" t="s">
+      <c r="E7" s="11" t="s">
         <v>98</v>
       </c>
-      <c r="F7" s="21"/>
-    </row>
-    <row r="8" spans="1:7" ht="14.4" x14ac:dyDescent="0.25">
-      <c r="A8" s="15"/>
-      <c r="B8" s="18"/>
+      <c r="F7" s="19"/>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A8" s="21"/>
+      <c r="B8" s="14"/>
       <c r="C8" s="3" t="s">
         <v>14</v>
       </c>
@@ -1109,11 +1105,11 @@
       <c r="E8" s="5" t="s">
         <v>99</v>
       </c>
-      <c r="F8" s="21"/>
-    </row>
-    <row r="9" spans="1:7" ht="14.4" x14ac:dyDescent="0.25">
-      <c r="A9" s="15"/>
-      <c r="B9" s="18"/>
+      <c r="F8" s="19"/>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A9" s="21"/>
+      <c r="B9" s="14"/>
       <c r="C9" s="3" t="s">
         <v>15</v>
       </c>
@@ -1121,11 +1117,11 @@
       <c r="E9" s="5" t="s">
         <v>100</v>
       </c>
-      <c r="F9" s="21"/>
-    </row>
-    <row r="10" spans="1:7" ht="14.4" x14ac:dyDescent="0.25">
-      <c r="A10" s="16"/>
-      <c r="B10" s="19"/>
+      <c r="F9" s="19"/>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A10" s="17"/>
+      <c r="B10" s="15"/>
       <c r="C10" s="3" t="s">
         <v>16</v>
       </c>
@@ -1133,13 +1129,13 @@
       <c r="E10" s="5" t="s">
         <v>101</v>
       </c>
-      <c r="F10" s="22"/>
-    </row>
-    <row r="11" spans="1:7" ht="14.4" x14ac:dyDescent="0.25">
-      <c r="A11" s="14" t="s">
+      <c r="F10" s="20"/>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A11" s="16" t="s">
         <v>17</v>
       </c>
-      <c r="B11" s="17" t="s">
+      <c r="B11" s="13" t="s">
         <v>18</v>
       </c>
       <c r="C11" s="3" t="s">
@@ -1151,13 +1147,13 @@
       <c r="E11" s="6" t="s">
         <v>102</v>
       </c>
-      <c r="F11" s="20" t="s">
+      <c r="F11" s="18" t="s">
         <v>103</v>
       </c>
     </row>
-    <row r="12" spans="1:7" ht="14.4" x14ac:dyDescent="0.25">
-      <c r="A12" s="15"/>
-      <c r="B12" s="18"/>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A12" s="21"/>
+      <c r="B12" s="14"/>
       <c r="C12" s="3" t="s">
         <v>20</v>
       </c>
@@ -1165,11 +1161,11 @@
       <c r="E12" s="6" t="s">
         <v>104</v>
       </c>
-      <c r="F12" s="21"/>
-    </row>
-    <row r="13" spans="1:7" ht="14.4" x14ac:dyDescent="0.25">
-      <c r="A13" s="16"/>
-      <c r="B13" s="19"/>
+      <c r="F12" s="19"/>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A13" s="17"/>
+      <c r="B13" s="15"/>
       <c r="C13" s="3" t="s">
         <v>22</v>
       </c>
@@ -1179,14 +1175,14 @@
       <c r="E13" s="6" t="s">
         <v>105</v>
       </c>
-      <c r="F13" s="22"/>
-    </row>
-    <row r="14" spans="1:7" ht="14.4" x14ac:dyDescent="0.25">
-      <c r="A14" s="14" t="s">
+      <c r="F13" s="20"/>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A14" s="16" t="s">
         <v>24</v>
       </c>
-      <c r="B14" s="17" t="s">
-        <v>136</v>
+      <c r="B14" s="13" t="s">
+        <v>135</v>
       </c>
       <c r="C14" s="8" t="s">
         <v>75</v>
@@ -1197,13 +1193,13 @@
       <c r="E14" s="9" t="s">
         <v>106</v>
       </c>
-      <c r="F14" s="20" t="s">
+      <c r="F14" s="18" t="s">
         <v>107</v>
       </c>
     </row>
-    <row r="15" spans="1:7" ht="14.4" x14ac:dyDescent="0.25">
-      <c r="A15" s="15"/>
-      <c r="B15" s="18"/>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A15" s="21"/>
+      <c r="B15" s="14"/>
       <c r="C15" s="3" t="s">
         <v>25</v>
       </c>
@@ -1211,13 +1207,13 @@
         <v>23</v>
       </c>
       <c r="E15" s="9" t="s">
-        <v>135</v>
-      </c>
-      <c r="F15" s="21"/>
-    </row>
-    <row r="16" spans="1:7" ht="14.4" x14ac:dyDescent="0.25">
-      <c r="A16" s="15"/>
-      <c r="B16" s="18"/>
+        <v>134</v>
+      </c>
+      <c r="F15" s="19"/>
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.2">
+      <c r="A16" s="21"/>
+      <c r="B16" s="14"/>
       <c r="C16" s="3" t="s">
         <v>27</v>
       </c>
@@ -1227,11 +1223,11 @@
       <c r="E16" s="9" t="s">
         <v>108</v>
       </c>
-      <c r="F16" s="21"/>
-    </row>
-    <row r="17" spans="1:6" ht="14.4" x14ac:dyDescent="0.25">
-      <c r="A17" s="15"/>
-      <c r="B17" s="18"/>
+      <c r="F16" s="19"/>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A17" s="21"/>
+      <c r="B17" s="14"/>
       <c r="C17" s="3" t="s">
         <v>29</v>
       </c>
@@ -1241,11 +1237,11 @@
       <c r="E17" s="9" t="s">
         <v>109</v>
       </c>
-      <c r="F17" s="21"/>
-    </row>
-    <row r="18" spans="1:6" ht="14.4" x14ac:dyDescent="0.25">
-      <c r="A18" s="15"/>
-      <c r="B18" s="18"/>
+      <c r="F17" s="19"/>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A18" s="21"/>
+      <c r="B18" s="14"/>
       <c r="C18" s="3" t="s">
         <v>16</v>
       </c>
@@ -1255,11 +1251,11 @@
       <c r="E18" s="9" t="s">
         <v>110</v>
       </c>
-      <c r="F18" s="21"/>
-    </row>
-    <row r="19" spans="1:6" ht="14.4" x14ac:dyDescent="0.25">
-      <c r="A19" s="15"/>
-      <c r="B19" s="18"/>
+      <c r="F18" s="19"/>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A19" s="21"/>
+      <c r="B19" s="14"/>
       <c r="C19" s="3" t="s">
         <v>32</v>
       </c>
@@ -1269,11 +1265,11 @@
       <c r="E19" s="9" t="s">
         <v>111</v>
       </c>
-      <c r="F19" s="21"/>
-    </row>
-    <row r="20" spans="1:6" ht="14.4" x14ac:dyDescent="0.25">
-      <c r="A20" s="15"/>
-      <c r="B20" s="18"/>
+      <c r="F19" s="19"/>
+    </row>
+    <row r="20" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A20" s="21"/>
+      <c r="B20" s="14"/>
       <c r="C20" s="3" t="s">
         <v>34</v>
       </c>
@@ -1283,11 +1279,11 @@
       <c r="E20" s="9" t="s">
         <v>112</v>
       </c>
-      <c r="F20" s="21"/>
-    </row>
-    <row r="21" spans="1:6" ht="14.4" x14ac:dyDescent="0.25">
-      <c r="A21" s="15"/>
-      <c r="B21" s="18"/>
+      <c r="F20" s="19"/>
+    </row>
+    <row r="21" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A21" s="21"/>
+      <c r="B21" s="14"/>
       <c r="C21" s="3" t="s">
         <v>36</v>
       </c>
@@ -1297,11 +1293,11 @@
       <c r="E21" s="9" t="s">
         <v>113</v>
       </c>
-      <c r="F21" s="21"/>
-    </row>
-    <row r="22" spans="1:6" ht="14.4" x14ac:dyDescent="0.25">
-      <c r="A22" s="15"/>
-      <c r="B22" s="18"/>
+      <c r="F21" s="19"/>
+    </row>
+    <row r="22" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A22" s="21"/>
+      <c r="B22" s="14"/>
       <c r="C22" s="3" t="s">
         <v>38</v>
       </c>
@@ -1311,11 +1307,11 @@
       <c r="E22" s="9" t="s">
         <v>114</v>
       </c>
-      <c r="F22" s="21"/>
-    </row>
-    <row r="23" spans="1:6" ht="14.4" x14ac:dyDescent="0.25">
-      <c r="A23" s="15"/>
-      <c r="B23" s="18"/>
+      <c r="F22" s="19"/>
+    </row>
+    <row r="23" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A23" s="21"/>
+      <c r="B23" s="14"/>
       <c r="C23" s="3" t="s">
         <v>39</v>
       </c>
@@ -1325,11 +1321,11 @@
       <c r="E23" s="9" t="s">
         <v>113</v>
       </c>
-      <c r="F23" s="21"/>
-    </row>
-    <row r="24" spans="1:6" ht="14.4" x14ac:dyDescent="0.25">
-      <c r="A24" s="15"/>
-      <c r="B24" s="18"/>
+      <c r="F23" s="19"/>
+    </row>
+    <row r="24" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A24" s="21"/>
+      <c r="B24" s="14"/>
       <c r="C24" s="3" t="s">
         <v>41</v>
       </c>
@@ -1339,11 +1335,11 @@
       <c r="E24" s="9" t="s">
         <v>115</v>
       </c>
-      <c r="F24" s="21"/>
-    </row>
-    <row r="25" spans="1:6" ht="14.4" x14ac:dyDescent="0.25">
-      <c r="A25" s="15"/>
-      <c r="B25" s="18"/>
+      <c r="F24" s="19"/>
+    </row>
+    <row r="25" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A25" s="21"/>
+      <c r="B25" s="14"/>
       <c r="C25" s="3" t="s">
         <v>43</v>
       </c>
@@ -1353,11 +1349,11 @@
       <c r="E25" s="9" t="s">
         <v>116</v>
       </c>
-      <c r="F25" s="21"/>
-    </row>
-    <row r="26" spans="1:6" ht="14.4" x14ac:dyDescent="0.25">
-      <c r="A26" s="15"/>
-      <c r="B26" s="18"/>
+      <c r="F25" s="19"/>
+    </row>
+    <row r="26" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A26" s="21"/>
+      <c r="B26" s="14"/>
       <c r="C26" s="3" t="s">
         <v>45</v>
       </c>
@@ -1367,11 +1363,11 @@
       <c r="E26" s="9" t="s">
         <v>117</v>
       </c>
-      <c r="F26" s="21"/>
-    </row>
-    <row r="27" spans="1:6" ht="14.4" x14ac:dyDescent="0.25">
-      <c r="A27" s="15"/>
-      <c r="B27" s="19"/>
+      <c r="F26" s="19"/>
+    </row>
+    <row r="27" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A27" s="21"/>
+      <c r="B27" s="15"/>
       <c r="C27" s="3" t="s">
         <v>47</v>
       </c>
@@ -1381,11 +1377,11 @@
       <c r="E27" s="9" t="s">
         <v>118</v>
       </c>
-      <c r="F27" s="21"/>
-    </row>
-    <row r="28" spans="1:6" ht="14.4" x14ac:dyDescent="0.25">
-      <c r="A28" s="15"/>
-      <c r="B28" s="17" t="s">
+      <c r="F27" s="19"/>
+    </row>
+    <row r="28" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A28" s="21"/>
+      <c r="B28" s="13" t="s">
         <v>48</v>
       </c>
       <c r="C28" s="3" t="s">
@@ -1395,13 +1391,13 @@
         <v>77</v>
       </c>
       <c r="E28" s="5" t="s">
-        <v>119</v>
-      </c>
-      <c r="F28" s="21"/>
-    </row>
-    <row r="29" spans="1:6" ht="14.4" x14ac:dyDescent="0.25">
-      <c r="A29" s="15"/>
-      <c r="B29" s="18"/>
+        <v>139</v>
+      </c>
+      <c r="F28" s="19"/>
+    </row>
+    <row r="29" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A29" s="21"/>
+      <c r="B29" s="14"/>
       <c r="C29" s="3" t="s">
         <v>50</v>
       </c>
@@ -1409,13 +1405,13 @@
         <v>78</v>
       </c>
       <c r="E29" s="5" t="s">
-        <v>120</v>
-      </c>
-      <c r="F29" s="21"/>
-    </row>
-    <row r="30" spans="1:6" ht="14.4" x14ac:dyDescent="0.25">
-      <c r="A30" s="15"/>
-      <c r="B30" s="18"/>
+        <v>119</v>
+      </c>
+      <c r="F29" s="19"/>
+    </row>
+    <row r="30" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A30" s="21"/>
+      <c r="B30" s="14"/>
       <c r="C30" s="3" t="s">
         <v>51</v>
       </c>
@@ -1423,13 +1419,13 @@
         <v>79</v>
       </c>
       <c r="E30" s="5" t="s">
-        <v>121</v>
-      </c>
-      <c r="F30" s="21"/>
-    </row>
-    <row r="31" spans="1:6" ht="14.4" x14ac:dyDescent="0.25">
-      <c r="A31" s="16"/>
-      <c r="B31" s="19"/>
+        <v>120</v>
+      </c>
+      <c r="F30" s="19"/>
+    </row>
+    <row r="31" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A31" s="17"/>
+      <c r="B31" s="15"/>
       <c r="C31" s="3" t="s">
         <v>52</v>
       </c>
@@ -1437,15 +1433,15 @@
         <v>80</v>
       </c>
       <c r="E31" s="5" t="s">
-        <v>122</v>
-      </c>
-      <c r="F31" s="22"/>
-    </row>
-    <row r="32" spans="1:6" ht="14.4" x14ac:dyDescent="0.25">
-      <c r="A32" s="14" t="s">
+        <v>121</v>
+      </c>
+      <c r="F31" s="20"/>
+    </row>
+    <row r="32" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A32" s="16" t="s">
         <v>53</v>
       </c>
-      <c r="B32" s="10" t="s">
+      <c r="B32" s="5" t="s">
         <v>54</v>
       </c>
       <c r="C32" s="3" t="s">
@@ -1455,83 +1451,83 @@
       <c r="E32" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="F32" s="20" t="s">
+      <c r="F32" s="18" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="33" spans="1:6" ht="14.4" x14ac:dyDescent="0.25">
-      <c r="A33" s="16"/>
-      <c r="B33" s="10" t="s">
+    <row r="33" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A33" s="17"/>
+      <c r="B33" s="5" t="s">
         <v>56</v>
       </c>
       <c r="C33" s="3" t="s">
+        <v>136</v>
+      </c>
+      <c r="D33" s="4"/>
+      <c r="E33" s="12" t="s">
+        <v>140</v>
+      </c>
+      <c r="F33" s="20"/>
+    </row>
+    <row r="34" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A34" s="16" t="s">
+        <v>57</v>
+      </c>
+      <c r="B34" s="13" t="s">
+        <v>58</v>
+      </c>
+      <c r="C34" s="3" t="s">
         <v>137</v>
       </c>
-      <c r="D33" s="4"/>
-      <c r="E33" s="23" t="s">
+      <c r="D34" s="4"/>
+      <c r="E34" s="12" t="s">
         <v>138</v>
       </c>
-      <c r="F33" s="22"/>
-    </row>
-    <row r="34" spans="1:6" ht="14.4" x14ac:dyDescent="0.25">
-      <c r="A34" s="14" t="s">
-        <v>57</v>
-      </c>
-      <c r="B34" s="17" t="s">
-        <v>58</v>
-      </c>
-      <c r="C34" s="3" t="s">
-        <v>139</v>
-      </c>
-      <c r="D34" s="4"/>
-      <c r="E34" s="23" t="s">
-        <v>140</v>
-      </c>
-      <c r="F34" s="20" t="s">
-        <v>123</v>
-      </c>
-    </row>
-    <row r="35" spans="1:6" ht="14.4" x14ac:dyDescent="0.25">
-      <c r="A35" s="15"/>
-      <c r="B35" s="18"/>
+      <c r="F34" s="18" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="35" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A35" s="21"/>
+      <c r="B35" s="14"/>
       <c r="C35" s="3" t="s">
         <v>59</v>
       </c>
       <c r="D35" s="4"/>
-      <c r="E35" s="13" t="s">
+      <c r="E35" s="11" t="s">
         <v>97</v>
       </c>
-      <c r="F35" s="21"/>
-    </row>
-    <row r="36" spans="1:6" ht="14.4" x14ac:dyDescent="0.25">
-      <c r="A36" s="15"/>
-      <c r="B36" s="18"/>
+      <c r="F35" s="19"/>
+    </row>
+    <row r="36" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A36" s="21"/>
+      <c r="B36" s="14"/>
       <c r="C36" s="3" t="s">
         <v>60</v>
       </c>
       <c r="D36" s="7"/>
-      <c r="E36" s="13" t="s">
+      <c r="E36" s="11" t="s">
         <v>98</v>
       </c>
-      <c r="F36" s="21"/>
-    </row>
-    <row r="37" spans="1:6" ht="14.4" x14ac:dyDescent="0.25">
-      <c r="A37" s="15"/>
-      <c r="B37" s="19"/>
+      <c r="F36" s="19"/>
+    </row>
+    <row r="37" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A37" s="21"/>
+      <c r="B37" s="15"/>
       <c r="C37" s="3" t="s">
         <v>62</v>
       </c>
       <c r="D37" s="4" t="s">
         <v>61</v>
       </c>
-      <c r="E37" s="13" t="s">
-        <v>124</v>
-      </c>
-      <c r="F37" s="21"/>
-    </row>
-    <row r="38" spans="1:6" ht="14.4" x14ac:dyDescent="0.25">
-      <c r="A38" s="15"/>
-      <c r="B38" s="17" t="s">
+      <c r="E37" s="11" t="s">
+        <v>123</v>
+      </c>
+      <c r="F37" s="19"/>
+    </row>
+    <row r="38" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A38" s="21"/>
+      <c r="B38" s="13" t="s">
         <v>64</v>
       </c>
       <c r="C38" s="3" t="s">
@@ -1541,13 +1537,13 @@
         <v>63</v>
       </c>
       <c r="E38" s="6" t="s">
-        <v>125</v>
-      </c>
-      <c r="F38" s="21"/>
-    </row>
-    <row r="39" spans="1:6" ht="14.4" x14ac:dyDescent="0.25">
-      <c r="A39" s="15"/>
-      <c r="B39" s="18"/>
+        <v>124</v>
+      </c>
+      <c r="F38" s="19"/>
+    </row>
+    <row r="39" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A39" s="21"/>
+      <c r="B39" s="14"/>
       <c r="C39" s="3" t="s">
         <v>67</v>
       </c>
@@ -1555,41 +1551,41 @@
         <v>66</v>
       </c>
       <c r="E39" s="6" t="s">
-        <v>126</v>
-      </c>
-      <c r="F39" s="21"/>
-    </row>
-    <row r="40" spans="1:6" ht="14.4" x14ac:dyDescent="0.25">
-      <c r="A40" s="15"/>
-      <c r="B40" s="18"/>
+        <v>125</v>
+      </c>
+      <c r="F39" s="19"/>
+    </row>
+    <row r="40" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A40" s="21"/>
+      <c r="B40" s="14"/>
       <c r="C40" s="3" t="s">
         <v>81</v>
       </c>
       <c r="D40" s="4" t="s">
         <v>82</v>
       </c>
-      <c r="E40" s="13" t="s">
-        <v>127</v>
-      </c>
-      <c r="F40" s="21"/>
-    </row>
-    <row r="41" spans="1:6" ht="14.4" x14ac:dyDescent="0.25">
-      <c r="A41" s="15"/>
-      <c r="B41" s="19"/>
+      <c r="E40" s="11" t="s">
+        <v>126</v>
+      </c>
+      <c r="F40" s="19"/>
+    </row>
+    <row r="41" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A41" s="21"/>
+      <c r="B41" s="15"/>
       <c r="C41" s="3" t="s">
         <v>83</v>
       </c>
       <c r="D41" s="4" t="s">
         <v>84</v>
       </c>
-      <c r="E41" s="13" t="s">
-        <v>128</v>
-      </c>
-      <c r="F41" s="21"/>
-    </row>
-    <row r="42" spans="1:6" ht="14.4" x14ac:dyDescent="0.25">
-      <c r="A42" s="15"/>
-      <c r="B42" s="17" t="s">
+      <c r="E41" s="11" t="s">
+        <v>127</v>
+      </c>
+      <c r="F41" s="19"/>
+    </row>
+    <row r="42" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A42" s="21"/>
+      <c r="B42" s="13" t="s">
         <v>68</v>
       </c>
       <c r="C42" s="3" t="s">
@@ -1599,13 +1595,13 @@
         <v>85</v>
       </c>
       <c r="E42" s="6" t="s">
-        <v>129</v>
-      </c>
-      <c r="F42" s="21"/>
-    </row>
-    <row r="43" spans="1:6" ht="14.4" x14ac:dyDescent="0.25">
-      <c r="A43" s="15"/>
-      <c r="B43" s="18"/>
+        <v>128</v>
+      </c>
+      <c r="F42" s="19"/>
+    </row>
+    <row r="43" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A43" s="21"/>
+      <c r="B43" s="14"/>
       <c r="C43" s="3" t="s">
         <v>69</v>
       </c>
@@ -1613,13 +1609,13 @@
         <v>86</v>
       </c>
       <c r="E43" s="6" t="s">
-        <v>130</v>
-      </c>
-      <c r="F43" s="21"/>
-    </row>
-    <row r="44" spans="1:6" ht="14.4" x14ac:dyDescent="0.25">
-      <c r="A44" s="15"/>
-      <c r="B44" s="18"/>
+        <v>129</v>
+      </c>
+      <c r="F43" s="19"/>
+    </row>
+    <row r="44" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A44" s="21"/>
+      <c r="B44" s="14"/>
       <c r="C44" s="3" t="s">
         <v>74</v>
       </c>
@@ -1627,13 +1623,13 @@
         <v>87</v>
       </c>
       <c r="E44" s="6" t="s">
-        <v>131</v>
-      </c>
-      <c r="F44" s="21"/>
-    </row>
-    <row r="45" spans="1:6" ht="14.4" x14ac:dyDescent="0.25">
-      <c r="A45" s="15"/>
-      <c r="B45" s="18"/>
+        <v>130</v>
+      </c>
+      <c r="F44" s="19"/>
+    </row>
+    <row r="45" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A45" s="21"/>
+      <c r="B45" s="14"/>
       <c r="C45" s="3" t="s">
         <v>91</v>
       </c>
@@ -1641,13 +1637,13 @@
         <v>92</v>
       </c>
       <c r="E45" s="6" t="s">
-        <v>132</v>
-      </c>
-      <c r="F45" s="21"/>
-    </row>
-    <row r="46" spans="1:6" ht="14.4" x14ac:dyDescent="0.25">
-      <c r="A46" s="15"/>
-      <c r="B46" s="18"/>
+        <v>131</v>
+      </c>
+      <c r="F45" s="19"/>
+    </row>
+    <row r="46" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A46" s="21"/>
+      <c r="B46" s="14"/>
       <c r="C46" s="3" t="s">
         <v>90</v>
       </c>
@@ -1655,13 +1651,13 @@
         <v>88</v>
       </c>
       <c r="E46" s="6" t="s">
-        <v>133</v>
-      </c>
-      <c r="F46" s="21"/>
-    </row>
-    <row r="47" spans="1:6" ht="14.4" x14ac:dyDescent="0.25">
-      <c r="A47" s="16"/>
-      <c r="B47" s="19"/>
+        <v>132</v>
+      </c>
+      <c r="F46" s="19"/>
+    </row>
+    <row r="47" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A47" s="17"/>
+      <c r="B47" s="15"/>
       <c r="C47" s="3" t="s">
         <v>70</v>
       </c>
@@ -1669,12 +1665,18 @@
         <v>89</v>
       </c>
       <c r="E47" s="6" t="s">
-        <v>134</v>
-      </c>
-      <c r="F47" s="22"/>
+        <v>133</v>
+      </c>
+      <c r="F47" s="20"/>
     </row>
   </sheetData>
   <mergeCells count="17">
+    <mergeCell ref="A2:A10"/>
+    <mergeCell ref="B2:B10"/>
+    <mergeCell ref="A11:A13"/>
+    <mergeCell ref="B11:B13"/>
+    <mergeCell ref="F2:F10"/>
+    <mergeCell ref="F11:F13"/>
     <mergeCell ref="B28:B31"/>
     <mergeCell ref="A32:A33"/>
     <mergeCell ref="F14:F31"/>
@@ -1686,12 +1688,6 @@
     <mergeCell ref="B42:B47"/>
     <mergeCell ref="A14:A31"/>
     <mergeCell ref="B14:B27"/>
-    <mergeCell ref="A2:A10"/>
-    <mergeCell ref="B2:B10"/>
-    <mergeCell ref="A11:A13"/>
-    <mergeCell ref="B11:B13"/>
-    <mergeCell ref="F2:F10"/>
-    <mergeCell ref="F11:F13"/>
   </mergeCells>
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
fix(export): fix error tips in excel file
fix error tips in excel file
</commit_message>
<xml_diff>
--- a/packages/api-server/assets/evaluation-template.xlsx
+++ b/packages/api-server/assets/evaluation-template.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Workspaces\Code\webProject\oss-evaluation-service\packages\api-server\assets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2A556DD7-DC56-42BD-B103-0F4391A39E1D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{30B69915-7487-4AD6-86B3-B091248D7F3D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -87,9 +87,6 @@
     <t>开发者满意度</t>
   </si>
   <si>
-    <t>代码量</t>
-  </si>
-  <si>
     <t>最佳实践评分基于Linux Foundation建议的Best Practices检查，每个检查项都有不同的权重</t>
   </si>
   <si>
@@ -361,9 +358,6 @@
     <t>&lt;%~_data_.evaluation.functionScore%&gt;</t>
   </si>
   <si>
-    <t>&lt;%~_data_.codeLines/1000%&gt; kl</t>
-  </si>
-  <si>
     <t>&lt;%~_data_.document.documentScore%&gt;</t>
   </si>
   <si>
@@ -476,6 +470,14 @@
   </si>
   <si>
     <t>&lt;%~_data_?.gzipSize/1024 || 'N/A' %&gt;</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>&lt;%~_data_.codeLines/1000%&gt;</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>代码量(kl)</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
 </sst>
@@ -1028,7 +1030,7 @@
       </c>
       <c r="D2" s="4"/>
       <c r="E2" s="5" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="F2" s="18" t="s">
         <v>7</v>
@@ -1043,7 +1045,7 @@
       </c>
       <c r="D3" s="4"/>
       <c r="E3" s="5" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="F3" s="19"/>
     </row>
@@ -1055,7 +1057,7 @@
       </c>
       <c r="D4" s="4"/>
       <c r="E4" s="4" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="F4" s="19"/>
     </row>
@@ -1067,7 +1069,7 @@
       </c>
       <c r="D5" s="4"/>
       <c r="E5" s="5" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="F5" s="19"/>
     </row>
@@ -1079,7 +1081,7 @@
       </c>
       <c r="D6" s="4"/>
       <c r="E6" s="11" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="F6" s="19"/>
     </row>
@@ -1091,7 +1093,7 @@
       </c>
       <c r="D7" s="4"/>
       <c r="E7" s="11" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="F7" s="19"/>
     </row>
@@ -1103,7 +1105,7 @@
       </c>
       <c r="D8" s="4"/>
       <c r="E8" s="5" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="F8" s="19"/>
     </row>
@@ -1115,7 +1117,7 @@
       </c>
       <c r="D9" s="4"/>
       <c r="E9" s="5" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="F9" s="19"/>
     </row>
@@ -1127,7 +1129,7 @@
       </c>
       <c r="D10" s="4"/>
       <c r="E10" s="5" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="F10" s="20"/>
     </row>
@@ -1142,24 +1144,24 @@
         <v>19</v>
       </c>
       <c r="D11" s="4" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="E11" s="6" t="s">
+        <v>101</v>
+      </c>
+      <c r="F11" s="18" t="s">
         <v>102</v>
-      </c>
-      <c r="F11" s="18" t="s">
-        <v>103</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A12" s="21"/>
       <c r="B12" s="14"/>
       <c r="C12" s="3" t="s">
-        <v>20</v>
+        <v>140</v>
       </c>
       <c r="D12" s="7"/>
       <c r="E12" s="6" t="s">
-        <v>104</v>
+        <v>139</v>
       </c>
       <c r="F12" s="19"/>
     </row>
@@ -1167,47 +1169,47 @@
       <c r="A13" s="17"/>
       <c r="B13" s="15"/>
       <c r="C13" s="3" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="D13" s="4" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="E13" s="6" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="F13" s="20"/>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A14" s="16" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B14" s="13" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="C14" s="8" t="s">
+        <v>74</v>
+      </c>
+      <c r="D14" s="4" t="s">
         <v>75</v>
       </c>
-      <c r="D14" s="4" t="s">
-        <v>76</v>
-      </c>
       <c r="E14" s="9" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="F14" s="18" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A15" s="21"/>
       <c r="B15" s="14"/>
       <c r="C15" s="3" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="D15" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="E15" s="9" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="F15" s="19"/>
     </row>
@@ -1215,13 +1217,13 @@
       <c r="A16" s="21"/>
       <c r="B16" s="14"/>
       <c r="C16" s="3" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="D16" s="4" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="E16" s="9" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="F16" s="19"/>
     </row>
@@ -1229,13 +1231,13 @@
       <c r="A17" s="21"/>
       <c r="B17" s="14"/>
       <c r="C17" s="3" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="D17" s="4" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="E17" s="9" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="F17" s="19"/>
     </row>
@@ -1246,10 +1248,10 @@
         <v>16</v>
       </c>
       <c r="D18" s="4" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="E18" s="9" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="F18" s="19"/>
     </row>
@@ -1257,13 +1259,13 @@
       <c r="A19" s="21"/>
       <c r="B19" s="14"/>
       <c r="C19" s="3" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="D19" s="4" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="E19" s="9" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="F19" s="19"/>
     </row>
@@ -1271,13 +1273,13 @@
       <c r="A20" s="21"/>
       <c r="B20" s="14"/>
       <c r="C20" s="3" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="D20" s="4" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="E20" s="9" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="F20" s="19"/>
     </row>
@@ -1285,13 +1287,13 @@
       <c r="A21" s="21"/>
       <c r="B21" s="14"/>
       <c r="C21" s="3" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="D21" s="4" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="E21" s="9" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="F21" s="19"/>
     </row>
@@ -1299,13 +1301,13 @@
       <c r="A22" s="21"/>
       <c r="B22" s="14"/>
       <c r="C22" s="3" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="D22" s="4" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="E22" s="9" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="F22" s="19"/>
     </row>
@@ -1313,13 +1315,13 @@
       <c r="A23" s="21"/>
       <c r="B23" s="14"/>
       <c r="C23" s="3" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="D23" s="4" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="E23" s="9" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="F23" s="19"/>
     </row>
@@ -1327,13 +1329,13 @@
       <c r="A24" s="21"/>
       <c r="B24" s="14"/>
       <c r="C24" s="3" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="D24" s="4" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="E24" s="9" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="F24" s="19"/>
     </row>
@@ -1341,13 +1343,13 @@
       <c r="A25" s="21"/>
       <c r="B25" s="14"/>
       <c r="C25" s="3" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="D25" s="4" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="E25" s="9" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="F25" s="19"/>
     </row>
@@ -1355,13 +1357,13 @@
       <c r="A26" s="21"/>
       <c r="B26" s="14"/>
       <c r="C26" s="3" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="D26" s="4" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="E26" s="9" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="F26" s="19"/>
     </row>
@@ -1369,29 +1371,29 @@
       <c r="A27" s="21"/>
       <c r="B27" s="15"/>
       <c r="C27" s="3" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="D27" s="4" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="E27" s="9" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="F27" s="19"/>
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A28" s="21"/>
       <c r="B28" s="13" t="s">
+        <v>47</v>
+      </c>
+      <c r="C28" s="3" t="s">
         <v>48</v>
       </c>
-      <c r="C28" s="3" t="s">
-        <v>49</v>
-      </c>
       <c r="D28" s="4" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="E28" s="5" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="F28" s="19"/>
     </row>
@@ -1399,13 +1401,13 @@
       <c r="A29" s="21"/>
       <c r="B29" s="14"/>
       <c r="C29" s="3" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="D29" s="4" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="E29" s="5" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="F29" s="19"/>
     </row>
@@ -1413,13 +1415,13 @@
       <c r="A30" s="21"/>
       <c r="B30" s="14"/>
       <c r="C30" s="3" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="D30" s="4" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="E30" s="5" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="F30" s="19"/>
     </row>
@@ -1427,25 +1429,25 @@
       <c r="A31" s="17"/>
       <c r="B31" s="15"/>
       <c r="C31" s="3" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="D31" s="4" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="E31" s="5" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="F31" s="20"/>
     </row>
     <row r="32" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A32" s="16" t="s">
+        <v>52</v>
+      </c>
+      <c r="B32" s="5" t="s">
         <v>53</v>
       </c>
-      <c r="B32" s="5" t="s">
+      <c r="C32" s="3" t="s">
         <v>54</v>
-      </c>
-      <c r="C32" s="3" t="s">
-        <v>55</v>
       </c>
       <c r="D32" s="4"/>
       <c r="E32" s="6" t="s">
@@ -1458,44 +1460,44 @@
     <row r="33" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A33" s="17"/>
       <c r="B33" s="5" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="C33" s="3" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="D33" s="4"/>
       <c r="E33" s="12" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="F33" s="20"/>
     </row>
     <row r="34" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A34" s="16" t="s">
+        <v>56</v>
+      </c>
+      <c r="B34" s="13" t="s">
         <v>57</v>
       </c>
-      <c r="B34" s="13" t="s">
-        <v>58</v>
-      </c>
       <c r="C34" s="3" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="D34" s="4"/>
       <c r="E34" s="12" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="F34" s="18" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
     </row>
     <row r="35" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A35" s="21"/>
       <c r="B35" s="14"/>
       <c r="C35" s="3" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="D35" s="4"/>
       <c r="E35" s="11" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="F35" s="19"/>
     </row>
@@ -1503,11 +1505,11 @@
       <c r="A36" s="21"/>
       <c r="B36" s="14"/>
       <c r="C36" s="3" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="D36" s="7"/>
       <c r="E36" s="11" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="F36" s="19"/>
     </row>
@@ -1515,29 +1517,29 @@
       <c r="A37" s="21"/>
       <c r="B37" s="15"/>
       <c r="C37" s="3" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="D37" s="4" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="E37" s="11" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="F37" s="19"/>
     </row>
     <row r="38" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A38" s="21"/>
       <c r="B38" s="13" t="s">
+        <v>63</v>
+      </c>
+      <c r="C38" s="3" t="s">
         <v>64</v>
       </c>
-      <c r="C38" s="3" t="s">
-        <v>65</v>
-      </c>
       <c r="D38" s="4" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="E38" s="6" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="F38" s="19"/>
     </row>
@@ -1545,13 +1547,13 @@
       <c r="A39" s="21"/>
       <c r="B39" s="14"/>
       <c r="C39" s="3" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="D39" s="4" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="E39" s="6" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="F39" s="19"/>
     </row>
@@ -1559,13 +1561,13 @@
       <c r="A40" s="21"/>
       <c r="B40" s="14"/>
       <c r="C40" s="3" t="s">
+        <v>80</v>
+      </c>
+      <c r="D40" s="4" t="s">
         <v>81</v>
       </c>
-      <c r="D40" s="4" t="s">
-        <v>82</v>
-      </c>
       <c r="E40" s="11" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="F40" s="19"/>
     </row>
@@ -1573,29 +1575,29 @@
       <c r="A41" s="21"/>
       <c r="B41" s="15"/>
       <c r="C41" s="3" t="s">
+        <v>82</v>
+      </c>
+      <c r="D41" s="4" t="s">
         <v>83</v>
       </c>
-      <c r="D41" s="4" t="s">
-        <v>84</v>
-      </c>
       <c r="E41" s="11" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="F41" s="19"/>
     </row>
     <row r="42" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A42" s="21"/>
       <c r="B42" s="13" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="C42" s="3" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="D42" s="4" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="E42" s="6" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="F42" s="19"/>
     </row>
@@ -1603,13 +1605,13 @@
       <c r="A43" s="21"/>
       <c r="B43" s="14"/>
       <c r="C43" s="3" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="D43" s="4" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="E43" s="6" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="F43" s="19"/>
     </row>
@@ -1617,13 +1619,13 @@
       <c r="A44" s="21"/>
       <c r="B44" s="14"/>
       <c r="C44" s="3" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="D44" s="4" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="E44" s="6" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="F44" s="19"/>
     </row>
@@ -1631,13 +1633,13 @@
       <c r="A45" s="21"/>
       <c r="B45" s="14"/>
       <c r="C45" s="3" t="s">
+        <v>90</v>
+      </c>
+      <c r="D45" s="4" t="s">
         <v>91</v>
       </c>
-      <c r="D45" s="4" t="s">
-        <v>92</v>
-      </c>
       <c r="E45" s="6" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="F45" s="19"/>
     </row>
@@ -1645,13 +1647,13 @@
       <c r="A46" s="21"/>
       <c r="B46" s="14"/>
       <c r="C46" s="3" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="D46" s="4" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="E46" s="6" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="F46" s="19"/>
     </row>
@@ -1659,13 +1661,13 @@
       <c r="A47" s="17"/>
       <c r="B47" s="15"/>
       <c r="C47" s="3" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="D47" s="4" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="E47" s="6" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="F47" s="20"/>
     </row>

</xml_diff>

<commit_message>
feat(export): add softwareCompare export api
add softwareCompare export api
</commit_message>
<xml_diff>
--- a/packages/api-server/assets/evaluation-template.xlsx
+++ b/packages/api-server/assets/evaluation-template.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27531"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="27830"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Workspaces\Code\webProject\oss-evaluation-service\packages\api-server\assets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{30B69915-7487-4AD6-86B3-B091248D7F3D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8EA51B93-71DE-48BA-85D4-F7D165E5A18D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="148" uniqueCount="141">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="148" uniqueCount="142">
   <si>
     <t>维度</t>
   </si>
@@ -478,6 +478,10 @@
   </si>
   <si>
     <t>代码量(kl)</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>&lt;%~_data_.scorecard.binaryArtifacts%&gt;</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
 </sst>
@@ -646,6 +650,15 @@
     <xf numFmtId="179" fontId="4" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -655,12 +668,6 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="176" fontId="4" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -668,9 +675,6 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="176" fontId="4" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1019,10 +1023,10 @@
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A2" s="16" t="s">
+      <c r="A2" s="13" t="s">
         <v>6</v>
       </c>
-      <c r="B2" s="13" t="s">
+      <c r="B2" s="16" t="s">
         <v>7</v>
       </c>
       <c r="C2" s="3" t="s">
@@ -1032,14 +1036,14 @@
       <c r="E2" s="5" t="s">
         <v>92</v>
       </c>
-      <c r="F2" s="18" t="s">
+      <c r="F2" s="19" t="s">
         <v>7</v>
       </c>
       <c r="G2" s="2"/>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A3" s="21"/>
-      <c r="B3" s="14"/>
+      <c r="A3" s="14"/>
+      <c r="B3" s="17"/>
       <c r="C3" s="3" t="s">
         <v>9</v>
       </c>
@@ -1047,11 +1051,11 @@
       <c r="E3" s="5" t="s">
         <v>93</v>
       </c>
-      <c r="F3" s="19"/>
+      <c r="F3" s="20"/>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A4" s="21"/>
-      <c r="B4" s="14"/>
+      <c r="A4" s="14"/>
+      <c r="B4" s="17"/>
       <c r="C4" s="3" t="s">
         <v>10</v>
       </c>
@@ -1059,11 +1063,11 @@
       <c r="E4" s="4" t="s">
         <v>94</v>
       </c>
-      <c r="F4" s="19"/>
+      <c r="F4" s="20"/>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A5" s="21"/>
-      <c r="B5" s="14"/>
+      <c r="A5" s="14"/>
+      <c r="B5" s="17"/>
       <c r="C5" s="3" t="s">
         <v>11</v>
       </c>
@@ -1071,11 +1075,11 @@
       <c r="E5" s="5" t="s">
         <v>95</v>
       </c>
-      <c r="F5" s="19"/>
+      <c r="F5" s="20"/>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A6" s="21"/>
-      <c r="B6" s="14"/>
+      <c r="A6" s="14"/>
+      <c r="B6" s="17"/>
       <c r="C6" s="3" t="s">
         <v>12</v>
       </c>
@@ -1083,11 +1087,11 @@
       <c r="E6" s="11" t="s">
         <v>96</v>
       </c>
-      <c r="F6" s="19"/>
+      <c r="F6" s="20"/>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A7" s="21"/>
-      <c r="B7" s="14"/>
+      <c r="A7" s="14"/>
+      <c r="B7" s="17"/>
       <c r="C7" s="3" t="s">
         <v>13</v>
       </c>
@@ -1095,11 +1099,11 @@
       <c r="E7" s="11" t="s">
         <v>97</v>
       </c>
-      <c r="F7" s="19"/>
+      <c r="F7" s="20"/>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A8" s="21"/>
-      <c r="B8" s="14"/>
+      <c r="A8" s="14"/>
+      <c r="B8" s="17"/>
       <c r="C8" s="3" t="s">
         <v>14</v>
       </c>
@@ -1107,11 +1111,11 @@
       <c r="E8" s="5" t="s">
         <v>98</v>
       </c>
-      <c r="F8" s="19"/>
+      <c r="F8" s="20"/>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A9" s="21"/>
-      <c r="B9" s="14"/>
+      <c r="A9" s="14"/>
+      <c r="B9" s="17"/>
       <c r="C9" s="3" t="s">
         <v>15</v>
       </c>
@@ -1119,11 +1123,11 @@
       <c r="E9" s="5" t="s">
         <v>99</v>
       </c>
-      <c r="F9" s="19"/>
+      <c r="F9" s="20"/>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A10" s="17"/>
-      <c r="B10" s="15"/>
+      <c r="A10" s="15"/>
+      <c r="B10" s="18"/>
       <c r="C10" s="3" t="s">
         <v>16</v>
       </c>
@@ -1131,13 +1135,13 @@
       <c r="E10" s="5" t="s">
         <v>100</v>
       </c>
-      <c r="F10" s="20"/>
+      <c r="F10" s="21"/>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A11" s="16" t="s">
+      <c r="A11" s="13" t="s">
         <v>17</v>
       </c>
-      <c r="B11" s="13" t="s">
+      <c r="B11" s="16" t="s">
         <v>18</v>
       </c>
       <c r="C11" s="3" t="s">
@@ -1149,13 +1153,13 @@
       <c r="E11" s="6" t="s">
         <v>101</v>
       </c>
-      <c r="F11" s="18" t="s">
+      <c r="F11" s="19" t="s">
         <v>102</v>
       </c>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A12" s="21"/>
-      <c r="B12" s="14"/>
+      <c r="A12" s="14"/>
+      <c r="B12" s="17"/>
       <c r="C12" s="3" t="s">
         <v>140</v>
       </c>
@@ -1163,11 +1167,11 @@
       <c r="E12" s="6" t="s">
         <v>139</v>
       </c>
-      <c r="F12" s="19"/>
+      <c r="F12" s="20"/>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A13" s="17"/>
-      <c r="B13" s="15"/>
+      <c r="A13" s="15"/>
+      <c r="B13" s="18"/>
       <c r="C13" s="3" t="s">
         <v>21</v>
       </c>
@@ -1177,13 +1181,13 @@
       <c r="E13" s="6" t="s">
         <v>103</v>
       </c>
-      <c r="F13" s="20"/>
+      <c r="F13" s="21"/>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A14" s="16" t="s">
+      <c r="A14" s="13" t="s">
         <v>23</v>
       </c>
-      <c r="B14" s="13" t="s">
+      <c r="B14" s="16" t="s">
         <v>133</v>
       </c>
       <c r="C14" s="8" t="s">
@@ -1195,13 +1199,13 @@
       <c r="E14" s="9" t="s">
         <v>104</v>
       </c>
-      <c r="F14" s="18" t="s">
+      <c r="F14" s="19" t="s">
         <v>105</v>
       </c>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A15" s="21"/>
-      <c r="B15" s="14"/>
+      <c r="A15" s="14"/>
+      <c r="B15" s="17"/>
       <c r="C15" s="3" t="s">
         <v>24</v>
       </c>
@@ -1211,11 +1215,11 @@
       <c r="E15" s="9" t="s">
         <v>132</v>
       </c>
-      <c r="F15" s="19"/>
+      <c r="F15" s="20"/>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.2">
-      <c r="A16" s="21"/>
-      <c r="B16" s="14"/>
+      <c r="A16" s="14"/>
+      <c r="B16" s="17"/>
       <c r="C16" s="3" t="s">
         <v>26</v>
       </c>
@@ -1225,11 +1229,11 @@
       <c r="E16" s="9" t="s">
         <v>106</v>
       </c>
-      <c r="F16" s="19"/>
+      <c r="F16" s="20"/>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A17" s="21"/>
-      <c r="B17" s="14"/>
+      <c r="A17" s="14"/>
+      <c r="B17" s="17"/>
       <c r="C17" s="3" t="s">
         <v>28</v>
       </c>
@@ -1239,11 +1243,11 @@
       <c r="E17" s="9" t="s">
         <v>107</v>
       </c>
-      <c r="F17" s="19"/>
+      <c r="F17" s="20"/>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A18" s="21"/>
-      <c r="B18" s="14"/>
+      <c r="A18" s="14"/>
+      <c r="B18" s="17"/>
       <c r="C18" s="3" t="s">
         <v>16</v>
       </c>
@@ -1253,11 +1257,11 @@
       <c r="E18" s="9" t="s">
         <v>108</v>
       </c>
-      <c r="F18" s="19"/>
+      <c r="F18" s="20"/>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A19" s="21"/>
-      <c r="B19" s="14"/>
+      <c r="A19" s="14"/>
+      <c r="B19" s="17"/>
       <c r="C19" s="3" t="s">
         <v>31</v>
       </c>
@@ -1267,11 +1271,11 @@
       <c r="E19" s="9" t="s">
         <v>109</v>
       </c>
-      <c r="F19" s="19"/>
+      <c r="F19" s="20"/>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A20" s="21"/>
-      <c r="B20" s="14"/>
+      <c r="A20" s="14"/>
+      <c r="B20" s="17"/>
       <c r="C20" s="3" t="s">
         <v>33</v>
       </c>
@@ -1281,11 +1285,11 @@
       <c r="E20" s="9" t="s">
         <v>110</v>
       </c>
-      <c r="F20" s="19"/>
+      <c r="F20" s="20"/>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A21" s="21"/>
-      <c r="B21" s="14"/>
+      <c r="A21" s="14"/>
+      <c r="B21" s="17"/>
       <c r="C21" s="3" t="s">
         <v>35</v>
       </c>
@@ -1295,11 +1299,11 @@
       <c r="E21" s="9" t="s">
         <v>111</v>
       </c>
-      <c r="F21" s="19"/>
+      <c r="F21" s="20"/>
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A22" s="21"/>
-      <c r="B22" s="14"/>
+      <c r="A22" s="14"/>
+      <c r="B22" s="17"/>
       <c r="C22" s="3" t="s">
         <v>37</v>
       </c>
@@ -1309,11 +1313,11 @@
       <c r="E22" s="9" t="s">
         <v>112</v>
       </c>
-      <c r="F22" s="19"/>
+      <c r="F22" s="20"/>
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A23" s="21"/>
-      <c r="B23" s="14"/>
+      <c r="A23" s="14"/>
+      <c r="B23" s="17"/>
       <c r="C23" s="3" t="s">
         <v>38</v>
       </c>
@@ -1321,13 +1325,13 @@
         <v>70</v>
       </c>
       <c r="E23" s="9" t="s">
-        <v>111</v>
-      </c>
-      <c r="F23" s="19"/>
+        <v>141</v>
+      </c>
+      <c r="F23" s="20"/>
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A24" s="21"/>
-      <c r="B24" s="14"/>
+      <c r="A24" s="14"/>
+      <c r="B24" s="17"/>
       <c r="C24" s="3" t="s">
         <v>40</v>
       </c>
@@ -1337,11 +1341,11 @@
       <c r="E24" s="9" t="s">
         <v>113</v>
       </c>
-      <c r="F24" s="19"/>
+      <c r="F24" s="20"/>
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A25" s="21"/>
-      <c r="B25" s="14"/>
+      <c r="A25" s="14"/>
+      <c r="B25" s="17"/>
       <c r="C25" s="3" t="s">
         <v>42</v>
       </c>
@@ -1351,11 +1355,11 @@
       <c r="E25" s="9" t="s">
         <v>114</v>
       </c>
-      <c r="F25" s="19"/>
+      <c r="F25" s="20"/>
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A26" s="21"/>
-      <c r="B26" s="14"/>
+      <c r="A26" s="14"/>
+      <c r="B26" s="17"/>
       <c r="C26" s="3" t="s">
         <v>44</v>
       </c>
@@ -1365,11 +1369,11 @@
       <c r="E26" s="9" t="s">
         <v>115</v>
       </c>
-      <c r="F26" s="19"/>
+      <c r="F26" s="20"/>
     </row>
     <row r="27" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A27" s="21"/>
-      <c r="B27" s="15"/>
+      <c r="A27" s="14"/>
+      <c r="B27" s="18"/>
       <c r="C27" s="3" t="s">
         <v>46</v>
       </c>
@@ -1379,11 +1383,11 @@
       <c r="E27" s="9" t="s">
         <v>116</v>
       </c>
-      <c r="F27" s="19"/>
+      <c r="F27" s="20"/>
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A28" s="21"/>
-      <c r="B28" s="13" t="s">
+      <c r="A28" s="14"/>
+      <c r="B28" s="16" t="s">
         <v>47</v>
       </c>
       <c r="C28" s="3" t="s">
@@ -1395,11 +1399,11 @@
       <c r="E28" s="5" t="s">
         <v>137</v>
       </c>
-      <c r="F28" s="19"/>
+      <c r="F28" s="20"/>
     </row>
     <row r="29" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A29" s="21"/>
-      <c r="B29" s="14"/>
+      <c r="A29" s="14"/>
+      <c r="B29" s="17"/>
       <c r="C29" s="3" t="s">
         <v>49</v>
       </c>
@@ -1409,11 +1413,11 @@
       <c r="E29" s="5" t="s">
         <v>117</v>
       </c>
-      <c r="F29" s="19"/>
+      <c r="F29" s="20"/>
     </row>
     <row r="30" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A30" s="21"/>
-      <c r="B30" s="14"/>
+      <c r="A30" s="14"/>
+      <c r="B30" s="17"/>
       <c r="C30" s="3" t="s">
         <v>50</v>
       </c>
@@ -1423,11 +1427,11 @@
       <c r="E30" s="5" t="s">
         <v>118</v>
       </c>
-      <c r="F30" s="19"/>
+      <c r="F30" s="20"/>
     </row>
     <row r="31" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A31" s="17"/>
-      <c r="B31" s="15"/>
+      <c r="A31" s="15"/>
+      <c r="B31" s="18"/>
       <c r="C31" s="3" t="s">
         <v>51</v>
       </c>
@@ -1437,10 +1441,10 @@
       <c r="E31" s="5" t="s">
         <v>119</v>
       </c>
-      <c r="F31" s="20"/>
+      <c r="F31" s="21"/>
     </row>
     <row r="32" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A32" s="16" t="s">
+      <c r="A32" s="13" t="s">
         <v>52</v>
       </c>
       <c r="B32" s="5" t="s">
@@ -1453,12 +1457,12 @@
       <c r="E32" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="F32" s="18" t="s">
+      <c r="F32" s="19" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="33" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A33" s="17"/>
+      <c r="A33" s="15"/>
       <c r="B33" s="5" t="s">
         <v>55</v>
       </c>
@@ -1469,13 +1473,13 @@
       <c r="E33" s="12" t="s">
         <v>138</v>
       </c>
-      <c r="F33" s="20"/>
+      <c r="F33" s="21"/>
     </row>
     <row r="34" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A34" s="16" t="s">
+      <c r="A34" s="13" t="s">
         <v>56</v>
       </c>
-      <c r="B34" s="13" t="s">
+      <c r="B34" s="16" t="s">
         <v>57</v>
       </c>
       <c r="C34" s="3" t="s">
@@ -1485,13 +1489,13 @@
       <c r="E34" s="12" t="s">
         <v>136</v>
       </c>
-      <c r="F34" s="18" t="s">
+      <c r="F34" s="19" t="s">
         <v>120</v>
       </c>
     </row>
     <row r="35" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A35" s="21"/>
-      <c r="B35" s="14"/>
+      <c r="A35" s="14"/>
+      <c r="B35" s="17"/>
       <c r="C35" s="3" t="s">
         <v>58</v>
       </c>
@@ -1499,11 +1503,11 @@
       <c r="E35" s="11" t="s">
         <v>96</v>
       </c>
-      <c r="F35" s="19"/>
+      <c r="F35" s="20"/>
     </row>
     <row r="36" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A36" s="21"/>
-      <c r="B36" s="14"/>
+      <c r="A36" s="14"/>
+      <c r="B36" s="17"/>
       <c r="C36" s="3" t="s">
         <v>59</v>
       </c>
@@ -1511,11 +1515,11 @@
       <c r="E36" s="11" t="s">
         <v>97</v>
       </c>
-      <c r="F36" s="19"/>
+      <c r="F36" s="20"/>
     </row>
     <row r="37" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A37" s="21"/>
-      <c r="B37" s="15"/>
+      <c r="A37" s="14"/>
+      <c r="B37" s="18"/>
       <c r="C37" s="3" t="s">
         <v>61</v>
       </c>
@@ -1525,11 +1529,11 @@
       <c r="E37" s="11" t="s">
         <v>121</v>
       </c>
-      <c r="F37" s="19"/>
+      <c r="F37" s="20"/>
     </row>
     <row r="38" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A38" s="21"/>
-      <c r="B38" s="13" t="s">
+      <c r="A38" s="14"/>
+      <c r="B38" s="16" t="s">
         <v>63</v>
       </c>
       <c r="C38" s="3" t="s">
@@ -1541,11 +1545,11 @@
       <c r="E38" s="6" t="s">
         <v>122</v>
       </c>
-      <c r="F38" s="19"/>
+      <c r="F38" s="20"/>
     </row>
     <row r="39" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A39" s="21"/>
-      <c r="B39" s="14"/>
+      <c r="A39" s="14"/>
+      <c r="B39" s="17"/>
       <c r="C39" s="3" t="s">
         <v>66</v>
       </c>
@@ -1555,11 +1559,11 @@
       <c r="E39" s="6" t="s">
         <v>123</v>
       </c>
-      <c r="F39" s="19"/>
+      <c r="F39" s="20"/>
     </row>
     <row r="40" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A40" s="21"/>
-      <c r="B40" s="14"/>
+      <c r="A40" s="14"/>
+      <c r="B40" s="17"/>
       <c r="C40" s="3" t="s">
         <v>80</v>
       </c>
@@ -1569,11 +1573,11 @@
       <c r="E40" s="11" t="s">
         <v>124</v>
       </c>
-      <c r="F40" s="19"/>
+      <c r="F40" s="20"/>
     </row>
     <row r="41" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A41" s="21"/>
-      <c r="B41" s="15"/>
+      <c r="A41" s="14"/>
+      <c r="B41" s="18"/>
       <c r="C41" s="3" t="s">
         <v>82</v>
       </c>
@@ -1583,11 +1587,11 @@
       <c r="E41" s="11" t="s">
         <v>125</v>
       </c>
-      <c r="F41" s="19"/>
+      <c r="F41" s="20"/>
     </row>
     <row r="42" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A42" s="21"/>
-      <c r="B42" s="13" t="s">
+      <c r="A42" s="14"/>
+      <c r="B42" s="16" t="s">
         <v>67</v>
       </c>
       <c r="C42" s="3" t="s">
@@ -1599,11 +1603,11 @@
       <c r="E42" s="6" t="s">
         <v>126</v>
       </c>
-      <c r="F42" s="19"/>
+      <c r="F42" s="20"/>
     </row>
     <row r="43" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A43" s="21"/>
-      <c r="B43" s="14"/>
+      <c r="A43" s="14"/>
+      <c r="B43" s="17"/>
       <c r="C43" s="3" t="s">
         <v>68</v>
       </c>
@@ -1613,11 +1617,11 @@
       <c r="E43" s="6" t="s">
         <v>127</v>
       </c>
-      <c r="F43" s="19"/>
+      <c r="F43" s="20"/>
     </row>
     <row r="44" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A44" s="21"/>
-      <c r="B44" s="14"/>
+      <c r="A44" s="14"/>
+      <c r="B44" s="17"/>
       <c r="C44" s="3" t="s">
         <v>73</v>
       </c>
@@ -1627,11 +1631,11 @@
       <c r="E44" s="6" t="s">
         <v>128</v>
       </c>
-      <c r="F44" s="19"/>
+      <c r="F44" s="20"/>
     </row>
     <row r="45" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A45" s="21"/>
-      <c r="B45" s="14"/>
+      <c r="A45" s="14"/>
+      <c r="B45" s="17"/>
       <c r="C45" s="3" t="s">
         <v>90</v>
       </c>
@@ -1641,11 +1645,11 @@
       <c r="E45" s="6" t="s">
         <v>129</v>
       </c>
-      <c r="F45" s="19"/>
+      <c r="F45" s="20"/>
     </row>
     <row r="46" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A46" s="21"/>
-      <c r="B46" s="14"/>
+      <c r="A46" s="14"/>
+      <c r="B46" s="17"/>
       <c r="C46" s="3" t="s">
         <v>89</v>
       </c>
@@ -1655,11 +1659,11 @@
       <c r="E46" s="6" t="s">
         <v>130</v>
       </c>
-      <c r="F46" s="19"/>
+      <c r="F46" s="20"/>
     </row>
     <row r="47" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A47" s="17"/>
-      <c r="B47" s="15"/>
+      <c r="A47" s="15"/>
+      <c r="B47" s="18"/>
       <c r="C47" s="3" t="s">
         <v>69</v>
       </c>
@@ -1669,16 +1673,10 @@
       <c r="E47" s="6" t="s">
         <v>131</v>
       </c>
-      <c r="F47" s="20"/>
+      <c r="F47" s="21"/>
     </row>
   </sheetData>
   <mergeCells count="17">
-    <mergeCell ref="A2:A10"/>
-    <mergeCell ref="B2:B10"/>
-    <mergeCell ref="A11:A13"/>
-    <mergeCell ref="B11:B13"/>
-    <mergeCell ref="F2:F10"/>
-    <mergeCell ref="F11:F13"/>
     <mergeCell ref="B28:B31"/>
     <mergeCell ref="A32:A33"/>
     <mergeCell ref="F14:F31"/>
@@ -1690,6 +1688,12 @@
     <mergeCell ref="B42:B47"/>
     <mergeCell ref="A14:A31"/>
     <mergeCell ref="B14:B27"/>
+    <mergeCell ref="A2:A10"/>
+    <mergeCell ref="B2:B10"/>
+    <mergeCell ref="A11:A13"/>
+    <mergeCell ref="B11:B13"/>
+    <mergeCell ref="F2:F10"/>
+    <mergeCell ref="F11:F13"/>
   </mergeCells>
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>